<commit_message>
Added 3 Sep data
</commit_message>
<xml_diff>
--- a/Computed_Flux/all_fluxes.xlsx
+++ b/Computed_Flux/all_fluxes.xlsx
@@ -598,16 +598,16 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>45810</v>
+        <v>45901</v>
       </c>
       <c r="C14" t="n">
-        <v>887.972894054391</v>
+        <v>1642.20847750066</v>
       </c>
       <c r="D14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -615,10 +615,10 @@
         <v>6</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>45817</v>
+        <v>45810</v>
       </c>
       <c r="C15" t="n">
-        <v>3620.01402513419</v>
+        <v>887.972894054391</v>
       </c>
       <c r="D15" t="s">
         <v>7</v>
@@ -629,10 +629,10 @@
         <v>6</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>45826</v>
+        <v>45817</v>
       </c>
       <c r="C16" t="n">
-        <v>5848.12551989594</v>
+        <v>3620.01402513419</v>
       </c>
       <c r="D16" t="s">
         <v>7</v>
@@ -643,10 +643,10 @@
         <v>6</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>45835</v>
+        <v>45826</v>
       </c>
       <c r="C17" t="n">
-        <v>795.27107195837</v>
+        <v>5848.12551989594</v>
       </c>
       <c r="D17" t="s">
         <v>7</v>
@@ -657,10 +657,10 @@
         <v>6</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>45842</v>
+        <v>45835</v>
       </c>
       <c r="C18" t="n">
-        <v>2863.65866842687</v>
+        <v>795.27107195837</v>
       </c>
       <c r="D18" t="s">
         <v>7</v>
@@ -671,10 +671,10 @@
         <v>6</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>45849</v>
+        <v>45842</v>
       </c>
       <c r="C19" t="n">
-        <v>582.771258652471</v>
+        <v>2863.65866842687</v>
       </c>
       <c r="D19" t="s">
         <v>7</v>
@@ -685,10 +685,10 @@
         <v>6</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>45856</v>
+        <v>45849</v>
       </c>
       <c r="C20" t="n">
-        <v>3774.37460704209</v>
+        <v>582.771258652471</v>
       </c>
       <c r="D20" t="s">
         <v>7</v>
@@ -699,10 +699,10 @@
         <v>6</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>45863</v>
+        <v>45856</v>
       </c>
       <c r="C21" t="n">
-        <v>980.83008292323</v>
+        <v>3774.37460704209</v>
       </c>
       <c r="D21" t="s">
         <v>7</v>
@@ -713,10 +713,10 @@
         <v>6</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>45873</v>
+        <v>45863</v>
       </c>
       <c r="C22" t="n">
-        <v>3776.52151072127</v>
+        <v>980.83008292323</v>
       </c>
       <c r="D22" t="s">
         <v>7</v>
@@ -727,10 +727,10 @@
         <v>6</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>45880</v>
+        <v>45873</v>
       </c>
       <c r="C23" t="n">
-        <v>4118.93954141025</v>
+        <v>3776.52151072127</v>
       </c>
       <c r="D23" t="s">
         <v>7</v>
@@ -741,10 +741,10 @@
         <v>6</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>45887</v>
+        <v>45880</v>
       </c>
       <c r="C24" t="n">
-        <v>3648.23270392578</v>
+        <v>4118.93954141025</v>
       </c>
       <c r="D24" t="s">
         <v>7</v>
@@ -755,10 +755,10 @@
         <v>6</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>45894</v>
+        <v>45887</v>
       </c>
       <c r="C25" t="n">
-        <v>2828.4104784591</v>
+        <v>3648.23270392578</v>
       </c>
       <c r="D25" t="s">
         <v>7</v>
@@ -766,30 +766,30 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>45810</v>
+        <v>45894</v>
       </c>
       <c r="C26" t="n">
-        <v>1114.95841751639</v>
+        <v>2828.4104784591</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>45817</v>
+        <v>45901</v>
       </c>
       <c r="C27" t="n">
-        <v>3967.21046532345</v>
+        <v>1609.55976707164</v>
       </c>
       <c r="D27" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
@@ -797,10 +797,10 @@
         <v>8</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>45826</v>
+        <v>45810</v>
       </c>
       <c r="C28" t="n">
-        <v>3404.56710734529</v>
+        <v>1114.95841751639</v>
       </c>
       <c r="D28" t="s">
         <v>9</v>
@@ -811,10 +811,10 @@
         <v>8</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>45835</v>
+        <v>45817</v>
       </c>
       <c r="C29" t="n">
-        <v>1999.33410190424</v>
+        <v>3967.21046532345</v>
       </c>
       <c r="D29" t="s">
         <v>9</v>
@@ -825,10 +825,10 @@
         <v>8</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>45842</v>
+        <v>45826</v>
       </c>
       <c r="C30" t="n">
-        <v>529.656630645944</v>
+        <v>3404.56710734529</v>
       </c>
       <c r="D30" t="s">
         <v>9</v>
@@ -839,10 +839,10 @@
         <v>8</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>45849</v>
+        <v>45835</v>
       </c>
       <c r="C31" t="n">
-        <v>4816.73679818835</v>
+        <v>1999.33410190424</v>
       </c>
       <c r="D31" t="s">
         <v>9</v>
@@ -853,10 +853,10 @@
         <v>8</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>45856</v>
+        <v>45842</v>
       </c>
       <c r="C32" t="n">
-        <v>2193.24328610956</v>
+        <v>529.656630645944</v>
       </c>
       <c r="D32" t="s">
         <v>9</v>
@@ -867,10 +867,10 @@
         <v>8</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>45863</v>
+        <v>45849</v>
       </c>
       <c r="C33" t="n">
-        <v>3643.24026825053</v>
+        <v>4816.73679818835</v>
       </c>
       <c r="D33" t="s">
         <v>9</v>
@@ -881,10 +881,10 @@
         <v>8</v>
       </c>
       <c r="B34" s="1" t="n">
-        <v>45873</v>
+        <v>45856</v>
       </c>
       <c r="C34" t="n">
-        <v>3128.79369665423</v>
+        <v>2193.24328610956</v>
       </c>
       <c r="D34" t="s">
         <v>9</v>
@@ -895,10 +895,10 @@
         <v>8</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>45880</v>
+        <v>45863</v>
       </c>
       <c r="C35" t="n">
-        <v>4586.82933528355</v>
+        <v>3643.24026825053</v>
       </c>
       <c r="D35" t="s">
         <v>9</v>
@@ -909,10 +909,10 @@
         <v>8</v>
       </c>
       <c r="B36" s="1" t="n">
-        <v>45887</v>
+        <v>45873</v>
       </c>
       <c r="C36" t="n">
-        <v>3394.16343445068</v>
+        <v>3128.79369665423</v>
       </c>
       <c r="D36" t="s">
         <v>9</v>
@@ -923,10 +923,10 @@
         <v>8</v>
       </c>
       <c r="B37" s="1" t="n">
-        <v>45894</v>
+        <v>45880</v>
       </c>
       <c r="C37" t="n">
-        <v>2703.9092133905</v>
+        <v>4586.82933528355</v>
       </c>
       <c r="D37" t="s">
         <v>9</v>
@@ -934,44 +934,44 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B38" s="1" t="n">
-        <v>45810</v>
+        <v>45887</v>
       </c>
       <c r="C38" t="n">
-        <v>896.001226735543</v>
+        <v>3394.16343445068</v>
       </c>
       <c r="D38" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B39" s="1" t="n">
-        <v>45817</v>
+        <v>45894</v>
       </c>
       <c r="C39" t="n">
-        <v>2030.70030492232</v>
+        <v>2703.9092133905</v>
       </c>
       <c r="D39" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B40" s="1" t="n">
-        <v>45826</v>
+        <v>45901</v>
       </c>
       <c r="C40" t="n">
-        <v>7084.27944063735</v>
+        <v>1785.31900434777</v>
       </c>
       <c r="D40" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41">
@@ -979,10 +979,10 @@
         <v>10</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>45835</v>
+        <v>45810</v>
       </c>
       <c r="C41" t="n">
-        <v>911.65002482044</v>
+        <v>896.001226735543</v>
       </c>
       <c r="D41" t="s">
         <v>5</v>
@@ -993,10 +993,10 @@
         <v>10</v>
       </c>
       <c r="B42" s="1" t="n">
-        <v>45842</v>
+        <v>45817</v>
       </c>
       <c r="C42" t="n">
-        <v>923.42600524363</v>
+        <v>2030.70030492232</v>
       </c>
       <c r="D42" t="s">
         <v>5</v>
@@ -1007,10 +1007,10 @@
         <v>10</v>
       </c>
       <c r="B43" s="1" t="n">
-        <v>45849</v>
+        <v>45826</v>
       </c>
       <c r="C43" t="n">
-        <v>2298.37541327764</v>
+        <v>7084.27944063735</v>
       </c>
       <c r="D43" t="s">
         <v>5</v>
@@ -1021,10 +1021,10 @@
         <v>10</v>
       </c>
       <c r="B44" s="1" t="n">
-        <v>45856</v>
+        <v>45835</v>
       </c>
       <c r="C44" t="n">
-        <v>2548.92674654963</v>
+        <v>911.65002482044</v>
       </c>
       <c r="D44" t="s">
         <v>5</v>
@@ -1035,10 +1035,10 @@
         <v>10</v>
       </c>
       <c r="B45" s="1" t="n">
-        <v>45863</v>
+        <v>45842</v>
       </c>
       <c r="C45" t="n">
-        <v>2284.96228575287</v>
+        <v>923.42600524363</v>
       </c>
       <c r="D45" t="s">
         <v>5</v>
@@ -1049,10 +1049,10 @@
         <v>10</v>
       </c>
       <c r="B46" s="1" t="n">
-        <v>45873</v>
+        <v>45849</v>
       </c>
       <c r="C46" t="n">
-        <v>2405.49680671009</v>
+        <v>2298.37541327764</v>
       </c>
       <c r="D46" t="s">
         <v>5</v>
@@ -1063,10 +1063,10 @@
         <v>10</v>
       </c>
       <c r="B47" s="1" t="n">
-        <v>45880</v>
+        <v>45856</v>
       </c>
       <c r="C47" t="n">
-        <v>5789.58956490831</v>
+        <v>2548.92674654963</v>
       </c>
       <c r="D47" t="s">
         <v>5</v>
@@ -1077,10 +1077,10 @@
         <v>10</v>
       </c>
       <c r="B48" s="1" t="n">
-        <v>45887</v>
+        <v>45863</v>
       </c>
       <c r="C48" t="n">
-        <v>3313.54847929235</v>
+        <v>2284.96228575287</v>
       </c>
       <c r="D48" t="s">
         <v>5</v>
@@ -1091,10 +1091,10 @@
         <v>10</v>
       </c>
       <c r="B49" s="1" t="n">
-        <v>45894</v>
+        <v>45873</v>
       </c>
       <c r="C49" t="n">
-        <v>3187.1648559333</v>
+        <v>2405.49680671009</v>
       </c>
       <c r="D49" t="s">
         <v>5</v>
@@ -1102,58 +1102,58 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B50" s="1" t="n">
-        <v>45810</v>
+        <v>45880</v>
       </c>
       <c r="C50" t="n">
-        <v>605.276401347038</v>
+        <v>5789.58956490831</v>
       </c>
       <c r="D50" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B51" s="1" t="n">
-        <v>45817</v>
+        <v>45887</v>
       </c>
       <c r="C51" t="n">
-        <v>3254.15705318998</v>
+        <v>3313.54847929235</v>
       </c>
       <c r="D51" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B52" s="1" t="n">
-        <v>45826</v>
+        <v>45894</v>
       </c>
       <c r="C52" t="n">
-        <v>5494.93846571461</v>
+        <v>3187.1648559333</v>
       </c>
       <c r="D52" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B53" s="1" t="n">
-        <v>45835</v>
+        <v>45901</v>
       </c>
       <c r="C53" t="n">
-        <v>493.831746277201</v>
+        <v>1469.24426484684</v>
       </c>
       <c r="D53" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54">
@@ -1161,10 +1161,10 @@
         <v>11</v>
       </c>
       <c r="B54" s="1" t="n">
-        <v>45842</v>
+        <v>45810</v>
       </c>
       <c r="C54" t="n">
-        <v>1033.1066084577</v>
+        <v>605.276401347038</v>
       </c>
       <c r="D54" t="s">
         <v>7</v>
@@ -1175,10 +1175,10 @@
         <v>11</v>
       </c>
       <c r="B55" s="1" t="n">
-        <v>45849</v>
+        <v>45817</v>
       </c>
       <c r="C55" t="n">
-        <v>809.578051527371</v>
+        <v>3254.15705318998</v>
       </c>
       <c r="D55" t="s">
         <v>7</v>
@@ -1189,10 +1189,10 @@
         <v>11</v>
       </c>
       <c r="B56" s="1" t="n">
-        <v>45856</v>
+        <v>45826</v>
       </c>
       <c r="C56" t="n">
-        <v>2699.12605710809</v>
+        <v>5494.93846571461</v>
       </c>
       <c r="D56" t="s">
         <v>7</v>
@@ -1203,10 +1203,10 @@
         <v>11</v>
       </c>
       <c r="B57" s="1" t="n">
-        <v>45863</v>
+        <v>45835</v>
       </c>
       <c r="C57" t="n">
-        <v>1219.60301108964</v>
+        <v>493.831746277201</v>
       </c>
       <c r="D57" t="s">
         <v>7</v>
@@ -1217,10 +1217,10 @@
         <v>11</v>
       </c>
       <c r="B58" s="1" t="n">
-        <v>45873</v>
+        <v>45842</v>
       </c>
       <c r="C58" t="n">
-        <v>3429.90174797312</v>
+        <v>1033.1066084577</v>
       </c>
       <c r="D58" t="s">
         <v>7</v>
@@ -1231,10 +1231,10 @@
         <v>11</v>
       </c>
       <c r="B59" s="1" t="n">
-        <v>45880</v>
+        <v>45849</v>
       </c>
       <c r="C59" t="n">
-        <v>3447.29762872426</v>
+        <v>809.578051527371</v>
       </c>
       <c r="D59" t="s">
         <v>7</v>
@@ -1245,10 +1245,10 @@
         <v>11</v>
       </c>
       <c r="B60" s="1" t="n">
-        <v>45887</v>
+        <v>45856</v>
       </c>
       <c r="C60" t="n">
-        <v>2971.31194167402</v>
+        <v>2699.12605710809</v>
       </c>
       <c r="D60" t="s">
         <v>7</v>
@@ -1259,10 +1259,10 @@
         <v>11</v>
       </c>
       <c r="B61" s="1" t="n">
-        <v>45894</v>
+        <v>45863</v>
       </c>
       <c r="C61" t="n">
-        <v>2128.81048195735</v>
+        <v>1219.60301108964</v>
       </c>
       <c r="D61" t="s">
         <v>7</v>
@@ -1270,72 +1270,72 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B62" s="1" t="n">
-        <v>45810</v>
+        <v>45873</v>
       </c>
       <c r="C62" t="n">
-        <v>829.274264965441</v>
+        <v>3429.90174797312</v>
       </c>
       <c r="D62" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B63" s="1" t="n">
-        <v>45817</v>
+        <v>45880</v>
       </c>
       <c r="C63" t="n">
-        <v>2034.26328932924</v>
+        <v>3447.29762872426</v>
       </c>
       <c r="D63" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B64" s="1" t="n">
-        <v>45826</v>
+        <v>45887</v>
       </c>
       <c r="C64" t="n">
-        <v>3085.76309059706</v>
+        <v>2971.31194167402</v>
       </c>
       <c r="D64" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B65" s="1" t="n">
-        <v>45835</v>
+        <v>45894</v>
       </c>
       <c r="C65" t="n">
-        <v>2113.86708643315</v>
+        <v>2128.81048195735</v>
       </c>
       <c r="D65" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B66" s="1" t="n">
-        <v>45842</v>
+        <v>45901</v>
       </c>
       <c r="C66" t="n">
-        <v>1158.7597584648</v>
+        <v>1885.52718940828</v>
       </c>
       <c r="D66" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67">
@@ -1343,10 +1343,10 @@
         <v>12</v>
       </c>
       <c r="B67" s="1" t="n">
-        <v>45849</v>
+        <v>45810</v>
       </c>
       <c r="C67" t="n">
-        <v>3804.85995259262</v>
+        <v>829.274264965441</v>
       </c>
       <c r="D67" t="s">
         <v>9</v>
@@ -1357,10 +1357,10 @@
         <v>12</v>
       </c>
       <c r="B68" s="1" t="n">
-        <v>45856</v>
+        <v>45817</v>
       </c>
       <c r="C68" t="n">
-        <v>1889.8067251411</v>
+        <v>2034.26328932924</v>
       </c>
       <c r="D68" t="s">
         <v>9</v>
@@ -1371,10 +1371,10 @@
         <v>12</v>
       </c>
       <c r="B69" s="1" t="n">
-        <v>45863</v>
+        <v>45826</v>
       </c>
       <c r="C69" t="n">
-        <v>4061.45488430826</v>
+        <v>3085.76309059706</v>
       </c>
       <c r="D69" t="s">
         <v>9</v>
@@ -1385,10 +1385,10 @@
         <v>12</v>
       </c>
       <c r="B70" s="1" t="n">
-        <v>45873</v>
+        <v>45835</v>
       </c>
       <c r="C70" t="n">
-        <v>2808.60882816944</v>
+        <v>2113.86708643315</v>
       </c>
       <c r="D70" t="s">
         <v>9</v>
@@ -1399,10 +1399,10 @@
         <v>12</v>
       </c>
       <c r="B71" s="1" t="n">
-        <v>45880</v>
+        <v>45842</v>
       </c>
       <c r="C71" t="n">
-        <v>4334.8959831226</v>
+        <v>1158.7597584648</v>
       </c>
       <c r="D71" t="s">
         <v>9</v>
@@ -1413,10 +1413,10 @@
         <v>12</v>
       </c>
       <c r="B72" s="1" t="n">
-        <v>45887</v>
+        <v>45849</v>
       </c>
       <c r="C72" t="n">
-        <v>1799.96285583044</v>
+        <v>3804.85995259262</v>
       </c>
       <c r="D72" t="s">
         <v>9</v>
@@ -1427,10 +1427,10 @@
         <v>12</v>
       </c>
       <c r="B73" s="1" t="n">
-        <v>45894</v>
+        <v>45856</v>
       </c>
       <c r="C73" t="n">
-        <v>3245.54806926349</v>
+        <v>1889.8067251411</v>
       </c>
       <c r="D73" t="s">
         <v>9</v>
@@ -1438,86 +1438,86 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B74" s="1" t="n">
-        <v>45810</v>
+        <v>45863</v>
       </c>
       <c r="C74" t="n">
-        <v>926.247921016511</v>
+        <v>4061.45488430826</v>
       </c>
       <c r="D74" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B75" s="1" t="n">
-        <v>45817</v>
+        <v>45873</v>
       </c>
       <c r="C75" t="n">
-        <v>1013.90634494399</v>
+        <v>2808.60882816944</v>
       </c>
       <c r="D75" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B76" s="1" t="n">
-        <v>45826</v>
+        <v>45880</v>
       </c>
       <c r="C76" t="n">
-        <v>2492.6382352641</v>
+        <v>4334.8959831226</v>
       </c>
       <c r="D76" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B77" s="1" t="n">
-        <v>45835</v>
+        <v>45887</v>
       </c>
       <c r="C77" t="n">
-        <v>208.353459554264</v>
+        <v>1799.96285583044</v>
       </c>
       <c r="D77" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B78" s="1" t="n">
-        <v>45842</v>
+        <v>45894</v>
       </c>
       <c r="C78" t="n">
-        <v>642.842381753608</v>
+        <v>3245.54806926349</v>
       </c>
       <c r="D78" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B79" s="1" t="n">
-        <v>45849</v>
+        <v>45901</v>
       </c>
       <c r="C79" t="n">
-        <v>708.264946681898</v>
+        <v>1181.54431177802</v>
       </c>
       <c r="D79" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80">
@@ -1525,10 +1525,10 @@
         <v>13</v>
       </c>
       <c r="B80" s="1" t="n">
-        <v>45856</v>
+        <v>45810</v>
       </c>
       <c r="C80" t="n">
-        <v>1297.74874736552</v>
+        <v>926.247921016511</v>
       </c>
       <c r="D80" t="s">
         <v>5</v>
@@ -1539,10 +1539,10 @@
         <v>13</v>
       </c>
       <c r="B81" s="1" t="n">
-        <v>45863</v>
+        <v>45817</v>
       </c>
       <c r="C81" t="n">
-        <v>1282.98566492001</v>
+        <v>1013.90634494399</v>
       </c>
       <c r="D81" t="s">
         <v>5</v>
@@ -1553,10 +1553,10 @@
         <v>13</v>
       </c>
       <c r="B82" s="1" t="n">
-        <v>45873</v>
+        <v>45826</v>
       </c>
       <c r="C82" t="n">
-        <v>3039.25791166093</v>
+        <v>2492.6382352641</v>
       </c>
       <c r="D82" t="s">
         <v>5</v>
@@ -1567,10 +1567,10 @@
         <v>13</v>
       </c>
       <c r="B83" s="1" t="n">
-        <v>45880</v>
+        <v>45835</v>
       </c>
       <c r="C83" t="n">
-        <v>4775.20972744648</v>
+        <v>208.353459554264</v>
       </c>
       <c r="D83" t="s">
         <v>5</v>
@@ -1581,10 +1581,10 @@
         <v>13</v>
       </c>
       <c r="B84" s="1" t="n">
-        <v>45887</v>
+        <v>45842</v>
       </c>
       <c r="C84" t="n">
-        <v>2089.81926332235</v>
+        <v>642.842381753608</v>
       </c>
       <c r="D84" t="s">
         <v>5</v>
@@ -1595,10 +1595,10 @@
         <v>13</v>
       </c>
       <c r="B85" s="1" t="n">
-        <v>45894</v>
+        <v>45849</v>
       </c>
       <c r="C85" t="n">
-        <v>4752.47660961459</v>
+        <v>708.264946681898</v>
       </c>
       <c r="D85" t="s">
         <v>5</v>
@@ -1606,100 +1606,100 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B86" s="1" t="n">
-        <v>45810</v>
+        <v>45856</v>
       </c>
       <c r="C86" t="n">
-        <v>820.429289044661</v>
+        <v>1297.74874736552</v>
       </c>
       <c r="D86" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B87" s="1" t="n">
-        <v>45817</v>
+        <v>45863</v>
       </c>
       <c r="C87" t="n">
-        <v>4438.5887346754</v>
+        <v>1282.98566492001</v>
       </c>
       <c r="D87" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B88" s="1" t="n">
-        <v>45826</v>
+        <v>45873</v>
       </c>
       <c r="C88" t="n">
-        <v>3375.80821888685</v>
+        <v>3039.25791166093</v>
       </c>
       <c r="D88" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B89" s="1" t="n">
-        <v>45835</v>
+        <v>45880</v>
       </c>
       <c r="C89" t="n">
-        <v>783.186507035906</v>
+        <v>4775.20972744648</v>
       </c>
       <c r="D89" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B90" s="1" t="n">
-        <v>45842</v>
+        <v>45887</v>
       </c>
       <c r="C90" t="n">
-        <v>631.923814275014</v>
+        <v>2089.81926332235</v>
       </c>
       <c r="D90" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B91" s="1" t="n">
-        <v>45849</v>
+        <v>45894</v>
       </c>
       <c r="C91" t="n">
-        <v>1315.52124698387</v>
+        <v>4752.47660961459</v>
       </c>
       <c r="D91" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B92" s="1" t="n">
-        <v>45856</v>
+        <v>45901</v>
       </c>
       <c r="C92" t="n">
-        <v>2207.89437180403</v>
+        <v>1541.24223720587</v>
       </c>
       <c r="D92" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="93">
@@ -1707,10 +1707,10 @@
         <v>14</v>
       </c>
       <c r="B93" s="1" t="n">
-        <v>45863</v>
+        <v>45810</v>
       </c>
       <c r="C93" t="n">
-        <v>2258.29619366983</v>
+        <v>820.429289044661</v>
       </c>
       <c r="D93" t="s">
         <v>7</v>
@@ -1721,10 +1721,10 @@
         <v>14</v>
       </c>
       <c r="B94" s="1" t="n">
-        <v>45873</v>
+        <v>45817</v>
       </c>
       <c r="C94" t="n">
-        <v>3728.99958287456</v>
+        <v>4438.5887346754</v>
       </c>
       <c r="D94" t="s">
         <v>7</v>
@@ -1735,10 +1735,10 @@
         <v>14</v>
       </c>
       <c r="B95" s="1" t="n">
-        <v>45880</v>
+        <v>45826</v>
       </c>
       <c r="C95" t="n">
-        <v>3912.32265691079</v>
+        <v>3375.80821888685</v>
       </c>
       <c r="D95" t="s">
         <v>7</v>
@@ -1749,10 +1749,10 @@
         <v>14</v>
       </c>
       <c r="B96" s="1" t="n">
-        <v>45887</v>
+        <v>45835</v>
       </c>
       <c r="C96" t="n">
-        <v>3599.81922977165</v>
+        <v>783.186507035906</v>
       </c>
       <c r="D96" t="s">
         <v>7</v>
@@ -1763,10 +1763,10 @@
         <v>14</v>
       </c>
       <c r="B97" s="1" t="n">
-        <v>45894</v>
+        <v>45842</v>
       </c>
       <c r="C97" t="n">
-        <v>2913.7632567457</v>
+        <v>631.923814275014</v>
       </c>
       <c r="D97" t="s">
         <v>7</v>
@@ -1774,114 +1774,114 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B98" s="1" t="n">
-        <v>45810</v>
+        <v>45849</v>
       </c>
       <c r="C98" t="n">
-        <v>749.87306919933</v>
+        <v>1315.52124698387</v>
       </c>
       <c r="D98" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B99" s="1" t="n">
-        <v>45817</v>
+        <v>45856</v>
       </c>
       <c r="C99" t="n">
-        <v>4412.64180269369</v>
+        <v>2207.89437180403</v>
       </c>
       <c r="D99" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B100" s="1" t="n">
-        <v>45826</v>
+        <v>45863</v>
       </c>
       <c r="C100" t="n">
-        <v>6968.33616394737</v>
+        <v>2258.29619366983</v>
       </c>
       <c r="D100" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B101" s="1" t="n">
-        <v>45835</v>
+        <v>45873</v>
       </c>
       <c r="C101" t="n">
-        <v>1687.73157419569</v>
+        <v>3728.99958287456</v>
       </c>
       <c r="D101" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B102" s="1" t="n">
-        <v>45842</v>
+        <v>45880</v>
       </c>
       <c r="C102" t="n">
-        <v>761.833024239517</v>
+        <v>3912.32265691079</v>
       </c>
       <c r="D102" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B103" s="1" t="n">
-        <v>45849</v>
+        <v>45887</v>
       </c>
       <c r="C103" t="n">
-        <v>2588.80886828618</v>
+        <v>3599.81922977165</v>
       </c>
       <c r="D103" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B104" s="1" t="n">
-        <v>45856</v>
+        <v>45894</v>
       </c>
       <c r="C104" t="n">
-        <v>3605.2695200209</v>
+        <v>2913.7632567457</v>
       </c>
       <c r="D104" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B105" s="1" t="n">
-        <v>45863</v>
+        <v>45901</v>
       </c>
       <c r="C105" t="n">
-        <v>2464.37485564112</v>
+        <v>2488.12022404981</v>
       </c>
       <c r="D105" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="106">
@@ -1889,10 +1889,10 @@
         <v>15</v>
       </c>
       <c r="B106" s="1" t="n">
-        <v>45873</v>
+        <v>45810</v>
       </c>
       <c r="C106" t="n">
-        <v>3566.94051479447</v>
+        <v>749.87306919933</v>
       </c>
       <c r="D106" t="s">
         <v>9</v>
@@ -1903,10 +1903,10 @@
         <v>15</v>
       </c>
       <c r="B107" s="1" t="n">
-        <v>45880</v>
+        <v>45817</v>
       </c>
       <c r="C107" t="n">
-        <v>5545.11780891709</v>
+        <v>4412.64180269369</v>
       </c>
       <c r="D107" t="s">
         <v>9</v>
@@ -1917,10 +1917,10 @@
         <v>15</v>
       </c>
       <c r="B108" s="1" t="n">
-        <v>45887</v>
+        <v>45826</v>
       </c>
       <c r="C108" t="n">
-        <v>2723.46038359217</v>
+        <v>6968.33616394737</v>
       </c>
       <c r="D108" t="s">
         <v>9</v>
@@ -1931,10 +1931,10 @@
         <v>15</v>
       </c>
       <c r="B109" s="1" t="n">
-        <v>45894</v>
+        <v>45835</v>
       </c>
       <c r="C109" t="n">
-        <v>3638.2311832252</v>
+        <v>1687.73157419569</v>
       </c>
       <c r="D109" t="s">
         <v>9</v>
@@ -1942,128 +1942,128 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B110" s="1" t="n">
-        <v>45810</v>
+        <v>45842</v>
       </c>
       <c r="C110" t="n">
-        <v>654.622171815671</v>
+        <v>761.833024239517</v>
       </c>
       <c r="D110" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B111" s="1" t="n">
-        <v>45817</v>
+        <v>45849</v>
       </c>
       <c r="C111" t="n">
-        <v>836.306701729539</v>
+        <v>2588.80886828618</v>
       </c>
       <c r="D111" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B112" s="1" t="n">
-        <v>45826</v>
+        <v>45856</v>
       </c>
       <c r="C112" t="n">
-        <v>752.809303565924</v>
+        <v>3605.2695200209</v>
       </c>
       <c r="D112" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B113" s="1" t="n">
-        <v>45835</v>
+        <v>45863</v>
       </c>
       <c r="C113" t="n">
-        <v>361.937925301449</v>
+        <v>2464.37485564112</v>
       </c>
       <c r="D113" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B114" s="1" t="n">
-        <v>45842</v>
+        <v>45873</v>
       </c>
       <c r="C114" t="n">
-        <v>274.147297459927</v>
+        <v>3566.94051479447</v>
       </c>
       <c r="D114" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B115" s="1" t="n">
-        <v>45849</v>
+        <v>45880</v>
       </c>
       <c r="C115" t="n">
-        <v>638.156969539091</v>
+        <v>5545.11780891709</v>
       </c>
       <c r="D115" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B116" s="1" t="n">
-        <v>45856</v>
+        <v>45887</v>
       </c>
       <c r="C116" t="n">
-        <v>671.100601945576</v>
+        <v>2723.46038359217</v>
       </c>
       <c r="D116" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B117" s="1" t="n">
-        <v>45863</v>
+        <v>45894</v>
       </c>
       <c r="C117" t="n">
-        <v>1126.92089194702</v>
+        <v>3638.2311832252</v>
       </c>
       <c r="D117" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B118" s="1" t="n">
-        <v>45873</v>
+        <v>45901</v>
       </c>
       <c r="C118" t="n">
-        <v>1904.69958425363</v>
+        <v>1849.60594842151</v>
       </c>
       <c r="D118" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="119">
@@ -2071,10 +2071,10 @@
         <v>16</v>
       </c>
       <c r="B119" s="1" t="n">
-        <v>45880</v>
+        <v>45810</v>
       </c>
       <c r="C119" t="n">
-        <v>3800.93540490905</v>
+        <v>654.622171815671</v>
       </c>
       <c r="D119" t="s">
         <v>5</v>
@@ -2085,10 +2085,10 @@
         <v>16</v>
       </c>
       <c r="B120" s="1" t="n">
-        <v>45887</v>
+        <v>45817</v>
       </c>
       <c r="C120" t="n">
-        <v>2170.9732688459</v>
+        <v>836.306701729539</v>
       </c>
       <c r="D120" t="s">
         <v>5</v>
@@ -2099,10 +2099,10 @@
         <v>16</v>
       </c>
       <c r="B121" s="1" t="n">
-        <v>45894</v>
+        <v>45826</v>
       </c>
       <c r="C121" t="n">
-        <v>3307.44136835169</v>
+        <v>752.809303565924</v>
       </c>
       <c r="D121" t="s">
         <v>5</v>
@@ -2110,142 +2110,142 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B122" s="1" t="n">
-        <v>45810</v>
+        <v>45835</v>
       </c>
       <c r="C122" t="n">
-        <v>714.089199892923</v>
+        <v>361.937925301449</v>
       </c>
       <c r="D122" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B123" s="1" t="n">
-        <v>45817</v>
+        <v>45842</v>
       </c>
       <c r="C123" t="n">
-        <v>1332.31394460659</v>
+        <v>274.147297459927</v>
       </c>
       <c r="D123" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B124" s="1" t="n">
-        <v>45826</v>
+        <v>45849</v>
       </c>
       <c r="C124" t="n">
-        <v>1403.48926864965</v>
+        <v>638.156969539091</v>
       </c>
       <c r="D124" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B125" s="1" t="n">
-        <v>45835</v>
+        <v>45856</v>
       </c>
       <c r="C125" t="n">
-        <v>423.584800449672</v>
+        <v>671.100601945576</v>
       </c>
       <c r="D125" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B126" s="1" t="n">
-        <v>45842</v>
+        <v>45863</v>
       </c>
       <c r="C126" t="n">
-        <v>691.944631498715</v>
+        <v>1126.92089194702</v>
       </c>
       <c r="D126" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B127" s="1" t="n">
-        <v>45849</v>
+        <v>45873</v>
       </c>
       <c r="C127" t="n">
-        <v>1520.16740554049</v>
+        <v>1904.69958425363</v>
       </c>
       <c r="D127" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B128" s="1" t="n">
-        <v>45856</v>
+        <v>45880</v>
       </c>
       <c r="C128" t="n">
-        <v>1394.70386978331</v>
+        <v>3800.93540490905</v>
       </c>
       <c r="D128" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B129" s="1" t="n">
-        <v>45863</v>
+        <v>45887</v>
       </c>
       <c r="C129" t="n">
-        <v>1945.74582627245</v>
+        <v>2170.9732688459</v>
       </c>
       <c r="D129" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B130" s="1" t="n">
-        <v>45873</v>
+        <v>45894</v>
       </c>
       <c r="C130" t="n">
-        <v>2541.97761269932</v>
+        <v>3307.44136835169</v>
       </c>
       <c r="D130" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B131" s="1" t="n">
-        <v>45880</v>
+        <v>45901</v>
       </c>
       <c r="C131" t="n">
-        <v>3884.74955947511</v>
+        <v>988.497215490608</v>
       </c>
       <c r="D131" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="132">
@@ -2253,10 +2253,10 @@
         <v>17</v>
       </c>
       <c r="B132" s="1" t="n">
-        <v>45887</v>
+        <v>45810</v>
       </c>
       <c r="C132" t="n">
-        <v>1740.78269526192</v>
+        <v>714.089199892923</v>
       </c>
       <c r="D132" t="s">
         <v>7</v>
@@ -2267,10 +2267,10 @@
         <v>17</v>
       </c>
       <c r="B133" s="1" t="n">
-        <v>45894</v>
+        <v>45817</v>
       </c>
       <c r="C133" t="n">
-        <v>2505.19645489012</v>
+        <v>1332.31394460659</v>
       </c>
       <c r="D133" t="s">
         <v>7</v>
@@ -2278,156 +2278,156 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B134" s="1" t="n">
-        <v>45810</v>
+        <v>45826</v>
       </c>
       <c r="C134" t="n">
-        <v>397.290437761417</v>
+        <v>1403.48926864965</v>
       </c>
       <c r="D134" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B135" s="1" t="n">
-        <v>45817</v>
+        <v>45835</v>
       </c>
       <c r="C135" t="n">
-        <v>1926.90668700788</v>
+        <v>423.584800449672</v>
       </c>
       <c r="D135" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B136" s="1" t="n">
-        <v>45826</v>
+        <v>45842</v>
       </c>
       <c r="C136" t="n">
-        <v>3021.29841712424</v>
+        <v>691.944631498715</v>
       </c>
       <c r="D136" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B137" s="1" t="n">
-        <v>45835</v>
+        <v>45849</v>
       </c>
       <c r="C137" t="n">
-        <v>957.104912247124</v>
+        <v>1520.16740554049</v>
       </c>
       <c r="D137" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B138" s="1" t="n">
-        <v>45842</v>
+        <v>45856</v>
       </c>
       <c r="C138" t="n">
-        <v>1649.6084629323</v>
+        <v>1394.70386978331</v>
       </c>
       <c r="D138" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B139" s="1" t="n">
-        <v>45849</v>
+        <v>45863</v>
       </c>
       <c r="C139" t="n">
-        <v>1539.67899281552</v>
+        <v>1945.74582627245</v>
       </c>
       <c r="D139" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B140" s="1" t="n">
-        <v>45856</v>
+        <v>45873</v>
       </c>
       <c r="C140" t="n">
-        <v>2459.63795093809</v>
+        <v>2541.97761269932</v>
       </c>
       <c r="D140" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B141" s="1" t="n">
-        <v>45863</v>
+        <v>45880</v>
       </c>
       <c r="C141" t="n">
-        <v>1996.741477782</v>
+        <v>3884.74955947511</v>
       </c>
       <c r="D141" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B142" s="1" t="n">
-        <v>45873</v>
+        <v>45887</v>
       </c>
       <c r="C142" t="n">
-        <v>3847.37405848995</v>
+        <v>1740.78269526192</v>
       </c>
       <c r="D142" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B143" s="1" t="n">
-        <v>45880</v>
+        <v>45894</v>
       </c>
       <c r="C143" t="n">
-        <v>2828.98818979552</v>
+        <v>2505.19645489012</v>
       </c>
       <c r="D143" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B144" s="1" t="n">
-        <v>45887</v>
+        <v>45901</v>
       </c>
       <c r="C144" t="n">
-        <v>2591.30540522796</v>
+        <v>973.643220252498</v>
       </c>
       <c r="D144" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="145">
@@ -2435,10 +2435,10 @@
         <v>18</v>
       </c>
       <c r="B145" s="1" t="n">
-        <v>45894</v>
+        <v>45810</v>
       </c>
       <c r="C145" t="n">
-        <v>1495.1664275966</v>
+        <v>397.290437761417</v>
       </c>
       <c r="D145" t="s">
         <v>9</v>
@@ -2446,505 +2446,715 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B146" s="1" t="n">
-        <v>45810</v>
+        <v>45817</v>
       </c>
       <c r="C146" t="n">
-        <v>564.435194569703</v>
+        <v>1926.90668700788</v>
       </c>
       <c r="D146" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B147" s="1" t="n">
-        <v>45817</v>
+        <v>45826</v>
       </c>
       <c r="C147" t="n">
-        <v>1545.70814869222</v>
+        <v>3021.29841712424</v>
       </c>
       <c r="D147" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B148" s="1" t="n">
-        <v>45826</v>
+        <v>45835</v>
       </c>
       <c r="C148" t="n">
-        <v>3858.60188057439</v>
+        <v>957.104912247124</v>
       </c>
       <c r="D148" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B149" s="1" t="n">
-        <v>45835</v>
+        <v>45842</v>
       </c>
       <c r="C149" t="n">
-        <v>75.8890033270052</v>
+        <v>1649.6084629323</v>
       </c>
       <c r="D149" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B150" s="1" t="n">
-        <v>45842</v>
+        <v>45849</v>
       </c>
       <c r="C150" t="n">
-        <v>1607.81816898261</v>
+        <v>1539.67899281552</v>
       </c>
       <c r="D150" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B151" s="1" t="n">
-        <v>45849</v>
+        <v>45856</v>
       </c>
       <c r="C151" t="n">
-        <v>651.305214716471</v>
+        <v>2459.63795093809</v>
       </c>
       <c r="D151" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B152" s="1" t="n">
-        <v>45856</v>
+        <v>45863</v>
       </c>
       <c r="C152" t="n">
-        <v>3182.90047392644</v>
+        <v>1996.741477782</v>
       </c>
       <c r="D152" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B153" s="1" t="n">
-        <v>45863</v>
+        <v>45873</v>
       </c>
       <c r="C153" t="n">
-        <v>1054.40680471126</v>
+        <v>3847.37405848995</v>
       </c>
       <c r="D153" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B154" s="1" t="n">
-        <v>45873</v>
+        <v>45880</v>
       </c>
       <c r="C154" t="n">
-        <v>3589.214407389</v>
+        <v>2828.98818979552</v>
       </c>
       <c r="D154" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B155" s="1" t="n">
-        <v>45880</v>
+        <v>45887</v>
       </c>
       <c r="C155" t="n">
-        <v>2375.18299388371</v>
+        <v>2591.30540522796</v>
       </c>
       <c r="D155" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B156" s="1" t="n">
-        <v>45887</v>
+        <v>45894</v>
       </c>
       <c r="C156" t="n">
-        <v>2768.14096770644</v>
+        <v>1495.1664275966</v>
       </c>
       <c r="D156" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B157" s="1" t="n">
-        <v>45894</v>
+        <v>45901</v>
       </c>
       <c r="C157" t="n">
-        <v>1810.23398806605</v>
+        <v>1208.07345867435</v>
       </c>
       <c r="D157" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B158" s="1" t="n">
         <v>45810</v>
       </c>
       <c r="C158" t="n">
-        <v>447.392417911663</v>
+        <v>564.435194569703</v>
       </c>
       <c r="D158" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B159" s="1" t="n">
         <v>45817</v>
       </c>
       <c r="C159" t="n">
-        <v>2644.87800920049</v>
+        <v>1545.70814869222</v>
       </c>
       <c r="D159" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B160" s="1" t="n">
         <v>45826</v>
       </c>
       <c r="C160" t="n">
-        <v>2858.8009710539</v>
+        <v>3858.60188057439</v>
       </c>
       <c r="D160" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B161" s="1" t="n">
         <v>45835</v>
       </c>
       <c r="C161" t="n">
-        <v>763.112592784348</v>
+        <v>75.8890033270052</v>
       </c>
       <c r="D161" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B162" s="1" t="n">
         <v>45842</v>
       </c>
       <c r="C162" t="n">
-        <v>674.542028148127</v>
+        <v>1607.81816898261</v>
       </c>
       <c r="D162" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B163" s="1" t="n">
         <v>45849</v>
       </c>
       <c r="C163" t="n">
-        <v>1744.34596755931</v>
+        <v>651.305214716471</v>
       </c>
       <c r="D163" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B164" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="C164" t="n">
-        <v>1143.7372540643</v>
+        <v>3182.90047392644</v>
       </c>
       <c r="D164" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B165" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C165" t="n">
-        <v>2601.30753317707</v>
+        <v>1054.40680471126</v>
       </c>
       <c r="D165" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B166" s="1" t="n">
         <v>45873</v>
       </c>
       <c r="C166" t="n">
-        <v>2436.60825019887</v>
+        <v>3589.214407389</v>
       </c>
       <c r="D166" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B167" s="1" t="n">
         <v>45880</v>
       </c>
       <c r="C167" t="n">
-        <v>3629.61304883485</v>
+        <v>2375.18299388371</v>
       </c>
       <c r="D167" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B168" s="1" t="n">
         <v>45887</v>
       </c>
       <c r="C168" t="n">
-        <v>2475.83592992463</v>
+        <v>2768.14096770644</v>
       </c>
       <c r="D168" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B169" s="1" t="n">
         <v>45894</v>
       </c>
       <c r="C169" t="n">
-        <v>2279.65892583665</v>
+        <v>1810.23398806605</v>
       </c>
       <c r="D169" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B170" s="1" t="n">
-        <v>45810</v>
+        <v>45901</v>
       </c>
       <c r="C170" t="n">
-        <v>844.462537825576</v>
+        <v>2132.26773713034</v>
       </c>
       <c r="D170" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B171" s="1" t="n">
-        <v>45817</v>
+        <v>45810</v>
       </c>
       <c r="C171" t="n">
-        <v>2607.51843632838</v>
+        <v>447.392417911663</v>
       </c>
       <c r="D171" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B172" s="1" t="n">
-        <v>45826</v>
+        <v>45817</v>
       </c>
       <c r="C172" t="n">
-        <v>1205.84904980573</v>
+        <v>2644.87800920049</v>
       </c>
       <c r="D172" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B173" s="1" t="n">
-        <v>45835</v>
+        <v>45826</v>
       </c>
       <c r="C173" t="n">
-        <v>394.51261524864</v>
+        <v>2858.8009710539</v>
       </c>
       <c r="D173" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B174" s="1" t="n">
-        <v>45842</v>
+        <v>45835</v>
       </c>
       <c r="C174" t="n">
-        <v>296.790183728622</v>
+        <v>763.112592784348</v>
       </c>
       <c r="D174" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B175" s="1" t="n">
-        <v>45849</v>
+        <v>45842</v>
       </c>
       <c r="C175" t="n">
-        <v>1029.40856752812</v>
+        <v>674.542028148127</v>
       </c>
       <c r="D175" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B176" s="1" t="n">
-        <v>45856</v>
+        <v>45849</v>
       </c>
       <c r="C176" t="n">
-        <v>822.899413189293</v>
+        <v>1744.34596755931</v>
       </c>
       <c r="D176" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B177" s="1" t="n">
-        <v>45863</v>
+        <v>45856</v>
       </c>
       <c r="C177" t="n">
-        <v>1093.38451398619</v>
+        <v>1143.7372540643</v>
       </c>
       <c r="D177" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B178" s="1" t="n">
-        <v>45873</v>
+        <v>45863</v>
       </c>
       <c r="C178" t="n">
-        <v>2628.07482556948</v>
+        <v>2601.30753317707</v>
       </c>
       <c r="D178" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B179" s="1" t="n">
-        <v>45880</v>
+        <v>45873</v>
       </c>
       <c r="C179" t="n">
-        <v>2995.86132481368</v>
+        <v>2436.60825019887</v>
       </c>
       <c r="D179" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B180" s="1" t="n">
-        <v>45887</v>
+        <v>45880</v>
       </c>
       <c r="C180" t="n">
-        <v>2000.21497594218</v>
+        <v>3629.61304883485</v>
       </c>
       <c r="D180" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="s">
+        <v>20</v>
+      </c>
+      <c r="B181" s="1" t="n">
+        <v>45887</v>
+      </c>
+      <c r="C181" t="n">
+        <v>2475.83592992463</v>
+      </c>
+      <c r="D181" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="s">
+        <v>20</v>
+      </c>
+      <c r="B182" s="1" t="n">
+        <v>45894</v>
+      </c>
+      <c r="C182" t="n">
+        <v>2279.65892583665</v>
+      </c>
+      <c r="D182" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="s">
+        <v>20</v>
+      </c>
+      <c r="B183" s="1" t="n">
+        <v>45901</v>
+      </c>
+      <c r="C183" t="n">
+        <v>998.259977017587</v>
+      </c>
+      <c r="D183" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="s">
         <v>21</v>
       </c>
-      <c r="B181" s="1" t="n">
+      <c r="B184" s="1" t="n">
+        <v>45810</v>
+      </c>
+      <c r="C184" t="n">
+        <v>844.462537825576</v>
+      </c>
+      <c r="D184" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="s">
+        <v>21</v>
+      </c>
+      <c r="B185" s="1" t="n">
+        <v>45817</v>
+      </c>
+      <c r="C185" t="n">
+        <v>2607.51843632838</v>
+      </c>
+      <c r="D185" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="s">
+        <v>21</v>
+      </c>
+      <c r="B186" s="1" t="n">
+        <v>45826</v>
+      </c>
+      <c r="C186" t="n">
+        <v>1205.84904980573</v>
+      </c>
+      <c r="D186" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="s">
+        <v>21</v>
+      </c>
+      <c r="B187" s="1" t="n">
+        <v>45835</v>
+      </c>
+      <c r="C187" t="n">
+        <v>394.51261524864</v>
+      </c>
+      <c r="D187" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="s">
+        <v>21</v>
+      </c>
+      <c r="B188" s="1" t="n">
+        <v>45842</v>
+      </c>
+      <c r="C188" t="n">
+        <v>296.790183728622</v>
+      </c>
+      <c r="D188" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="s">
+        <v>21</v>
+      </c>
+      <c r="B189" s="1" t="n">
+        <v>45849</v>
+      </c>
+      <c r="C189" t="n">
+        <v>1029.40856752812</v>
+      </c>
+      <c r="D189" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="s">
+        <v>21</v>
+      </c>
+      <c r="B190" s="1" t="n">
+        <v>45856</v>
+      </c>
+      <c r="C190" t="n">
+        <v>822.899413189293</v>
+      </c>
+      <c r="D190" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="s">
+        <v>21</v>
+      </c>
+      <c r="B191" s="1" t="n">
+        <v>45863</v>
+      </c>
+      <c r="C191" t="n">
+        <v>1093.38451398619</v>
+      </c>
+      <c r="D191" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="s">
+        <v>21</v>
+      </c>
+      <c r="B192" s="1" t="n">
+        <v>45873</v>
+      </c>
+      <c r="C192" t="n">
+        <v>2628.07482556948</v>
+      </c>
+      <c r="D192" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="s">
+        <v>21</v>
+      </c>
+      <c r="B193" s="1" t="n">
+        <v>45880</v>
+      </c>
+      <c r="C193" t="n">
+        <v>2995.86132481368</v>
+      </c>
+      <c r="D193" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="s">
+        <v>21</v>
+      </c>
+      <c r="B194" s="1" t="n">
+        <v>45887</v>
+      </c>
+      <c r="C194" t="n">
+        <v>2000.21497594218</v>
+      </c>
+      <c r="D194" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="s">
+        <v>21</v>
+      </c>
+      <c r="B195" s="1" t="n">
         <v>45894</v>
       </c>
-      <c r="C181" t="n">
+      <c r="C195" t="n">
         <v>1879.36457990422</v>
       </c>
-      <c r="D181" t="s">
+      <c r="D195" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="s">
+        <v>21</v>
+      </c>
+      <c r="B196" s="1" t="n">
+        <v>45901</v>
+      </c>
+      <c r="C196" t="n">
+        <v>967.384492520583</v>
+      </c>
+      <c r="D196" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
computed final yields for 2025. interim cumulative CH4 using licor only data
</commit_message>
<xml_diff>
--- a/Computed_Flux/all_fluxes.xlsx
+++ b/Computed_Flux/all_fluxes.xlsx
@@ -612,44 +612,44 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>45810</v>
+        <v>45908</v>
       </c>
       <c r="C15" t="n">
-        <v>887.972894054391</v>
+        <v>825.497971906722</v>
       </c>
       <c r="D15" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>45817</v>
+        <v>45912</v>
       </c>
       <c r="C16" t="n">
-        <v>3620.01402513419</v>
+        <v>5094.94811274734</v>
       </c>
       <c r="D16" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>45826</v>
+        <v>45918</v>
       </c>
       <c r="C17" t="n">
-        <v>5848.12551989594</v>
+        <v>29.1384604509441</v>
       </c>
       <c r="D17" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -657,10 +657,10 @@
         <v>6</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>45835</v>
+        <v>45810</v>
       </c>
       <c r="C18" t="n">
-        <v>795.27107195837</v>
+        <v>887.972894054391</v>
       </c>
       <c r="D18" t="s">
         <v>7</v>
@@ -671,10 +671,10 @@
         <v>6</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>45842</v>
+        <v>45817</v>
       </c>
       <c r="C19" t="n">
-        <v>2863.65866842687</v>
+        <v>3620.01402513419</v>
       </c>
       <c r="D19" t="s">
         <v>7</v>
@@ -685,10 +685,10 @@
         <v>6</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>45849</v>
+        <v>45826</v>
       </c>
       <c r="C20" t="n">
-        <v>582.771258652471</v>
+        <v>5848.12551989594</v>
       </c>
       <c r="D20" t="s">
         <v>7</v>
@@ -699,10 +699,10 @@
         <v>6</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>45856</v>
+        <v>45835</v>
       </c>
       <c r="C21" t="n">
-        <v>3774.37460704209</v>
+        <v>795.27107195837</v>
       </c>
       <c r="D21" t="s">
         <v>7</v>
@@ -713,10 +713,10 @@
         <v>6</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>45863</v>
+        <v>45842</v>
       </c>
       <c r="C22" t="n">
-        <v>980.83008292323</v>
+        <v>2863.65866842687</v>
       </c>
       <c r="D22" t="s">
         <v>7</v>
@@ -727,10 +727,10 @@
         <v>6</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>45873</v>
+        <v>45849</v>
       </c>
       <c r="C23" t="n">
-        <v>3776.52151072127</v>
+        <v>582.771258652471</v>
       </c>
       <c r="D23" t="s">
         <v>7</v>
@@ -741,10 +741,10 @@
         <v>6</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>45880</v>
+        <v>45856</v>
       </c>
       <c r="C24" t="n">
-        <v>4118.93954141025</v>
+        <v>3774.37460704209</v>
       </c>
       <c r="D24" t="s">
         <v>7</v>
@@ -755,10 +755,10 @@
         <v>6</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>45887</v>
+        <v>45863</v>
       </c>
       <c r="C25" t="n">
-        <v>3648.23270392578</v>
+        <v>980.83008292323</v>
       </c>
       <c r="D25" t="s">
         <v>7</v>
@@ -769,10 +769,10 @@
         <v>6</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>45894</v>
+        <v>45873</v>
       </c>
       <c r="C26" t="n">
-        <v>2828.4104784591</v>
+        <v>3776.52151072127</v>
       </c>
       <c r="D26" t="s">
         <v>7</v>
@@ -783,10 +783,10 @@
         <v>6</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>45901</v>
+        <v>45880</v>
       </c>
       <c r="C27" t="n">
-        <v>1609.55976707164</v>
+        <v>4118.93954141025</v>
       </c>
       <c r="D27" t="s">
         <v>7</v>
@@ -794,86 +794,86 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>45810</v>
+        <v>45887</v>
       </c>
       <c r="C28" t="n">
-        <v>1114.95841751639</v>
+        <v>3648.23270392578</v>
       </c>
       <c r="D28" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>45817</v>
+        <v>45894</v>
       </c>
       <c r="C29" t="n">
-        <v>3967.21046532345</v>
+        <v>2828.4104784591</v>
       </c>
       <c r="D29" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>45826</v>
+        <v>45901</v>
       </c>
       <c r="C30" t="n">
-        <v>3404.56710734529</v>
+        <v>1609.55976707164</v>
       </c>
       <c r="D30" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>45835</v>
+        <v>45908</v>
       </c>
       <c r="C31" t="n">
-        <v>1999.33410190424</v>
+        <v>863.703280702658</v>
       </c>
       <c r="D31" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>45842</v>
+        <v>45912</v>
       </c>
       <c r="C32" t="n">
-        <v>529.656630645944</v>
+        <v>4204.24412434881</v>
       </c>
       <c r="D32" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>45849</v>
+        <v>45918</v>
       </c>
       <c r="C33" t="n">
-        <v>4816.73679818835</v>
+        <v>56.8832320221224</v>
       </c>
       <c r="D33" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -881,10 +881,10 @@
         <v>8</v>
       </c>
       <c r="B34" s="1" t="n">
-        <v>45856</v>
+        <v>45810</v>
       </c>
       <c r="C34" t="n">
-        <v>2193.24328610956</v>
+        <v>1114.95841751639</v>
       </c>
       <c r="D34" t="s">
         <v>9</v>
@@ -895,10 +895,10 @@
         <v>8</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>45863</v>
+        <v>45817</v>
       </c>
       <c r="C35" t="n">
-        <v>3643.24026825053</v>
+        <v>3967.21046532345</v>
       </c>
       <c r="D35" t="s">
         <v>9</v>
@@ -909,10 +909,10 @@
         <v>8</v>
       </c>
       <c r="B36" s="1" t="n">
-        <v>45873</v>
+        <v>45826</v>
       </c>
       <c r="C36" t="n">
-        <v>3128.79369665423</v>
+        <v>3404.56710734529</v>
       </c>
       <c r="D36" t="s">
         <v>9</v>
@@ -923,10 +923,10 @@
         <v>8</v>
       </c>
       <c r="B37" s="1" t="n">
-        <v>45880</v>
+        <v>45835</v>
       </c>
       <c r="C37" t="n">
-        <v>4586.82933528355</v>
+        <v>1999.33410190424</v>
       </c>
       <c r="D37" t="s">
         <v>9</v>
@@ -937,10 +937,10 @@
         <v>8</v>
       </c>
       <c r="B38" s="1" t="n">
-        <v>45887</v>
+        <v>45842</v>
       </c>
       <c r="C38" t="n">
-        <v>3394.16343445068</v>
+        <v>529.656630645944</v>
       </c>
       <c r="D38" t="s">
         <v>9</v>
@@ -951,10 +951,10 @@
         <v>8</v>
       </c>
       <c r="B39" s="1" t="n">
-        <v>45894</v>
+        <v>45849</v>
       </c>
       <c r="C39" t="n">
-        <v>2703.9092133905</v>
+        <v>4816.73679818835</v>
       </c>
       <c r="D39" t="s">
         <v>9</v>
@@ -965,10 +965,10 @@
         <v>8</v>
       </c>
       <c r="B40" s="1" t="n">
-        <v>45901</v>
+        <v>45856</v>
       </c>
       <c r="C40" t="n">
-        <v>1785.31900434777</v>
+        <v>2193.24328610956</v>
       </c>
       <c r="D40" t="s">
         <v>9</v>
@@ -976,128 +976,128 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>45810</v>
+        <v>45863</v>
       </c>
       <c r="C41" t="n">
-        <v>896.001226735543</v>
+        <v>3643.24026825053</v>
       </c>
       <c r="D41" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B42" s="1" t="n">
-        <v>45817</v>
+        <v>45873</v>
       </c>
       <c r="C42" t="n">
-        <v>2030.70030492232</v>
+        <v>3128.79369665423</v>
       </c>
       <c r="D42" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B43" s="1" t="n">
-        <v>45826</v>
+        <v>45880</v>
       </c>
       <c r="C43" t="n">
-        <v>7084.27944063735</v>
+        <v>4586.82933528355</v>
       </c>
       <c r="D43" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B44" s="1" t="n">
-        <v>45835</v>
+        <v>45887</v>
       </c>
       <c r="C44" t="n">
-        <v>911.65002482044</v>
+        <v>3394.16343445068</v>
       </c>
       <c r="D44" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B45" s="1" t="n">
-        <v>45842</v>
+        <v>45894</v>
       </c>
       <c r="C45" t="n">
-        <v>923.42600524363</v>
+        <v>2703.9092133905</v>
       </c>
       <c r="D45" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B46" s="1" t="n">
-        <v>45849</v>
+        <v>45901</v>
       </c>
       <c r="C46" t="n">
-        <v>2298.37541327764</v>
+        <v>1785.31900434777</v>
       </c>
       <c r="D46" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B47" s="1" t="n">
-        <v>45856</v>
+        <v>45908</v>
       </c>
       <c r="C47" t="n">
-        <v>2548.92674654963</v>
+        <v>4661.49033559175</v>
       </c>
       <c r="D47" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B48" s="1" t="n">
-        <v>45863</v>
+        <v>45912</v>
       </c>
       <c r="C48" t="n">
-        <v>2284.96228575287</v>
+        <v>1775.28253834679</v>
       </c>
       <c r="D48" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B49" s="1" t="n">
-        <v>45873</v>
+        <v>45918</v>
       </c>
       <c r="C49" t="n">
-        <v>2405.49680671009</v>
+        <v>16.58013358516</v>
       </c>
       <c r="D49" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="50">
@@ -1105,10 +1105,10 @@
         <v>10</v>
       </c>
       <c r="B50" s="1" t="n">
-        <v>45880</v>
+        <v>45810</v>
       </c>
       <c r="C50" t="n">
-        <v>5789.58956490831</v>
+        <v>896.001226735543</v>
       </c>
       <c r="D50" t="s">
         <v>5</v>
@@ -1119,10 +1119,10 @@
         <v>10</v>
       </c>
       <c r="B51" s="1" t="n">
-        <v>45887</v>
+        <v>45817</v>
       </c>
       <c r="C51" t="n">
-        <v>3313.54847929235</v>
+        <v>2030.70030492232</v>
       </c>
       <c r="D51" t="s">
         <v>5</v>
@@ -1133,10 +1133,10 @@
         <v>10</v>
       </c>
       <c r="B52" s="1" t="n">
-        <v>45894</v>
+        <v>45826</v>
       </c>
       <c r="C52" t="n">
-        <v>3187.1648559333</v>
+        <v>7084.27944063735</v>
       </c>
       <c r="D52" t="s">
         <v>5</v>
@@ -1147,10 +1147,10 @@
         <v>10</v>
       </c>
       <c r="B53" s="1" t="n">
-        <v>45901</v>
+        <v>45835</v>
       </c>
       <c r="C53" t="n">
-        <v>1469.24426484684</v>
+        <v>911.65002482044</v>
       </c>
       <c r="D53" t="s">
         <v>5</v>
@@ -1158,170 +1158,170 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B54" s="1" t="n">
-        <v>45810</v>
+        <v>45842</v>
       </c>
       <c r="C54" t="n">
-        <v>605.276401347038</v>
+        <v>923.42600524363</v>
       </c>
       <c r="D54" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B55" s="1" t="n">
-        <v>45817</v>
+        <v>45849</v>
       </c>
       <c r="C55" t="n">
-        <v>3254.15705318998</v>
+        <v>2298.37541327764</v>
       </c>
       <c r="D55" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B56" s="1" t="n">
-        <v>45826</v>
+        <v>45856</v>
       </c>
       <c r="C56" t="n">
-        <v>5494.93846571461</v>
+        <v>2548.92674654963</v>
       </c>
       <c r="D56" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B57" s="1" t="n">
-        <v>45835</v>
+        <v>45863</v>
       </c>
       <c r="C57" t="n">
-        <v>493.831746277201</v>
+        <v>2284.96228575287</v>
       </c>
       <c r="D57" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B58" s="1" t="n">
-        <v>45842</v>
+        <v>45873</v>
       </c>
       <c r="C58" t="n">
-        <v>1033.1066084577</v>
+        <v>2405.49680671009</v>
       </c>
       <c r="D58" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B59" s="1" t="n">
-        <v>45849</v>
+        <v>45880</v>
       </c>
       <c r="C59" t="n">
-        <v>809.578051527371</v>
+        <v>5789.58956490831</v>
       </c>
       <c r="D59" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B60" s="1" t="n">
-        <v>45856</v>
+        <v>45887</v>
       </c>
       <c r="C60" t="n">
-        <v>2699.12605710809</v>
+        <v>3313.54847929235</v>
       </c>
       <c r="D60" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B61" s="1" t="n">
-        <v>45863</v>
+        <v>45894</v>
       </c>
       <c r="C61" t="n">
-        <v>1219.60301108964</v>
+        <v>3187.1648559333</v>
       </c>
       <c r="D61" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B62" s="1" t="n">
-        <v>45873</v>
+        <v>45901</v>
       </c>
       <c r="C62" t="n">
-        <v>3429.90174797312</v>
+        <v>1469.24426484684</v>
       </c>
       <c r="D62" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B63" s="1" t="n">
-        <v>45880</v>
+        <v>45908</v>
       </c>
       <c r="C63" t="n">
-        <v>3447.29762872426</v>
+        <v>4410.13371410884</v>
       </c>
       <c r="D63" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B64" s="1" t="n">
-        <v>45887</v>
+        <v>45912</v>
       </c>
       <c r="C64" t="n">
-        <v>2971.31194167402</v>
+        <v>5088.9184064008</v>
       </c>
       <c r="D64" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B65" s="1" t="n">
-        <v>45894</v>
+        <v>45918</v>
       </c>
       <c r="C65" t="n">
-        <v>2128.81048195735</v>
+        <v>46.9554905447005</v>
       </c>
       <c r="D65" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66">
@@ -1329,10 +1329,10 @@
         <v>11</v>
       </c>
       <c r="B66" s="1" t="n">
-        <v>45901</v>
+        <v>45810</v>
       </c>
       <c r="C66" t="n">
-        <v>1885.52718940828</v>
+        <v>605.276401347038</v>
       </c>
       <c r="D66" t="s">
         <v>7</v>
@@ -1340,1105 +1340,1105 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B67" s="1" t="n">
-        <v>45810</v>
+        <v>45817</v>
       </c>
       <c r="C67" t="n">
-        <v>829.274264965441</v>
+        <v>3254.15705318998</v>
       </c>
       <c r="D67" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B68" s="1" t="n">
-        <v>45817</v>
+        <v>45826</v>
       </c>
       <c r="C68" t="n">
-        <v>2034.26328932924</v>
+        <v>5494.93846571461</v>
       </c>
       <c r="D68" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" s="1" t="n">
-        <v>45826</v>
+        <v>45835</v>
       </c>
       <c r="C69" t="n">
-        <v>3085.76309059706</v>
+        <v>493.831746277201</v>
       </c>
       <c r="D69" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B70" s="1" t="n">
-        <v>45835</v>
+        <v>45842</v>
       </c>
       <c r="C70" t="n">
-        <v>2113.86708643315</v>
+        <v>1033.1066084577</v>
       </c>
       <c r="D70" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B71" s="1" t="n">
-        <v>45842</v>
+        <v>45849</v>
       </c>
       <c r="C71" t="n">
-        <v>1158.7597584648</v>
+        <v>809.578051527371</v>
       </c>
       <c r="D71" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B72" s="1" t="n">
-        <v>45849</v>
+        <v>45856</v>
       </c>
       <c r="C72" t="n">
-        <v>3804.85995259262</v>
+        <v>2699.12605710809</v>
       </c>
       <c r="D72" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B73" s="1" t="n">
-        <v>45856</v>
+        <v>45863</v>
       </c>
       <c r="C73" t="n">
-        <v>1889.8067251411</v>
+        <v>1219.60301108964</v>
       </c>
       <c r="D73" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B74" s="1" t="n">
-        <v>45863</v>
+        <v>45873</v>
       </c>
       <c r="C74" t="n">
-        <v>4061.45488430826</v>
+        <v>3429.90174797312</v>
       </c>
       <c r="D74" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B75" s="1" t="n">
-        <v>45873</v>
+        <v>45880</v>
       </c>
       <c r="C75" t="n">
-        <v>2808.60882816944</v>
+        <v>3447.29762872426</v>
       </c>
       <c r="D75" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B76" s="1" t="n">
-        <v>45880</v>
+        <v>45887</v>
       </c>
       <c r="C76" t="n">
-        <v>4334.8959831226</v>
+        <v>2971.31194167402</v>
       </c>
       <c r="D76" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B77" s="1" t="n">
-        <v>45887</v>
+        <v>45894</v>
       </c>
       <c r="C77" t="n">
-        <v>1799.96285583044</v>
+        <v>2128.81048195735</v>
       </c>
       <c r="D77" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B78" s="1" t="n">
-        <v>45894</v>
+        <v>45901</v>
       </c>
       <c r="C78" t="n">
-        <v>3245.54806926349</v>
+        <v>1885.52718940828</v>
       </c>
       <c r="D78" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B79" s="1" t="n">
-        <v>45901</v>
+        <v>45908</v>
       </c>
       <c r="C79" t="n">
-        <v>1181.54431177802</v>
+        <v>955.895358696291</v>
       </c>
       <c r="D79" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B80" s="1" t="n">
-        <v>45810</v>
+        <v>45912</v>
       </c>
       <c r="C80" t="n">
-        <v>926.247921016511</v>
+        <v>4439.99904036154</v>
       </c>
       <c r="D80" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B81" s="1" t="n">
-        <v>45817</v>
+        <v>45918</v>
       </c>
       <c r="C81" t="n">
-        <v>1013.90634494399</v>
+        <v>39.7251409513983</v>
       </c>
       <c r="D81" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B82" s="1" t="n">
-        <v>45826</v>
+        <v>45810</v>
       </c>
       <c r="C82" t="n">
-        <v>2492.6382352641</v>
+        <v>829.274264965441</v>
       </c>
       <c r="D82" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B83" s="1" t="n">
-        <v>45835</v>
+        <v>45817</v>
       </c>
       <c r="C83" t="n">
-        <v>208.353459554264</v>
+        <v>2034.26328932924</v>
       </c>
       <c r="D83" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B84" s="1" t="n">
-        <v>45842</v>
+        <v>45826</v>
       </c>
       <c r="C84" t="n">
-        <v>642.842381753608</v>
+        <v>3085.76309059706</v>
       </c>
       <c r="D84" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B85" s="1" t="n">
-        <v>45849</v>
+        <v>45835</v>
       </c>
       <c r="C85" t="n">
-        <v>708.264946681898</v>
+        <v>2113.86708643315</v>
       </c>
       <c r="D85" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B86" s="1" t="n">
-        <v>45856</v>
+        <v>45842</v>
       </c>
       <c r="C86" t="n">
-        <v>1297.74874736552</v>
+        <v>1158.7597584648</v>
       </c>
       <c r="D86" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B87" s="1" t="n">
-        <v>45863</v>
+        <v>45849</v>
       </c>
       <c r="C87" t="n">
-        <v>1282.98566492001</v>
+        <v>3804.85995259262</v>
       </c>
       <c r="D87" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B88" s="1" t="n">
-        <v>45873</v>
+        <v>45856</v>
       </c>
       <c r="C88" t="n">
-        <v>3039.25791166093</v>
+        <v>1889.8067251411</v>
       </c>
       <c r="D88" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B89" s="1" t="n">
-        <v>45880</v>
+        <v>45863</v>
       </c>
       <c r="C89" t="n">
-        <v>4775.20972744648</v>
+        <v>4061.45488430826</v>
       </c>
       <c r="D89" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B90" s="1" t="n">
-        <v>45887</v>
+        <v>45873</v>
       </c>
       <c r="C90" t="n">
-        <v>2089.81926332235</v>
+        <v>2808.60882816944</v>
       </c>
       <c r="D90" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B91" s="1" t="n">
-        <v>45894</v>
+        <v>45880</v>
       </c>
       <c r="C91" t="n">
-        <v>4752.47660961459</v>
+        <v>4334.8959831226</v>
       </c>
       <c r="D91" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B92" s="1" t="n">
-        <v>45901</v>
+        <v>45887</v>
       </c>
       <c r="C92" t="n">
-        <v>1541.24223720587</v>
+        <v>1799.96285583044</v>
       </c>
       <c r="D92" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B93" s="1" t="n">
-        <v>45810</v>
+        <v>45894</v>
       </c>
       <c r="C93" t="n">
-        <v>820.429289044661</v>
+        <v>3245.54806926349</v>
       </c>
       <c r="D93" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B94" s="1" t="n">
-        <v>45817</v>
+        <v>45901</v>
       </c>
       <c r="C94" t="n">
-        <v>4438.5887346754</v>
+        <v>1181.54431177802</v>
       </c>
       <c r="D94" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B95" s="1" t="n">
-        <v>45826</v>
+        <v>45908</v>
       </c>
       <c r="C95" t="n">
-        <v>3375.80821888685</v>
+        <v>1565.61592820745</v>
       </c>
       <c r="D95" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B96" s="1" t="n">
-        <v>45835</v>
+        <v>45912</v>
       </c>
       <c r="C96" t="n">
-        <v>783.186507035906</v>
+        <v>1461.3157191967</v>
       </c>
       <c r="D96" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B97" s="1" t="n">
-        <v>45842</v>
+        <v>45918</v>
       </c>
       <c r="C97" t="n">
-        <v>631.923814275014</v>
+        <v>31.2360864618781</v>
       </c>
       <c r="D97" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B98" s="1" t="n">
-        <v>45849</v>
+        <v>45810</v>
       </c>
       <c r="C98" t="n">
-        <v>1315.52124698387</v>
+        <v>926.247921016511</v>
       </c>
       <c r="D98" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B99" s="1" t="n">
-        <v>45856</v>
+        <v>45817</v>
       </c>
       <c r="C99" t="n">
-        <v>2207.89437180403</v>
+        <v>1013.90634494399</v>
       </c>
       <c r="D99" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B100" s="1" t="n">
-        <v>45863</v>
+        <v>45826</v>
       </c>
       <c r="C100" t="n">
-        <v>2258.29619366983</v>
+        <v>2492.6382352641</v>
       </c>
       <c r="D100" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B101" s="1" t="n">
-        <v>45873</v>
+        <v>45835</v>
       </c>
       <c r="C101" t="n">
-        <v>3728.99958287456</v>
+        <v>208.353459554264</v>
       </c>
       <c r="D101" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B102" s="1" t="n">
-        <v>45880</v>
+        <v>45842</v>
       </c>
       <c r="C102" t="n">
-        <v>3912.32265691079</v>
+        <v>642.842381753608</v>
       </c>
       <c r="D102" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B103" s="1" t="n">
-        <v>45887</v>
+        <v>45849</v>
       </c>
       <c r="C103" t="n">
-        <v>3599.81922977165</v>
+        <v>708.264946681898</v>
       </c>
       <c r="D103" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B104" s="1" t="n">
-        <v>45894</v>
+        <v>45856</v>
       </c>
       <c r="C104" t="n">
-        <v>2913.7632567457</v>
+        <v>1297.74874736552</v>
       </c>
       <c r="D104" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B105" s="1" t="n">
-        <v>45901</v>
+        <v>45863</v>
       </c>
       <c r="C105" t="n">
-        <v>2488.12022404981</v>
+        <v>1282.98566492001</v>
       </c>
       <c r="D105" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B106" s="1" t="n">
-        <v>45810</v>
+        <v>45873</v>
       </c>
       <c r="C106" t="n">
-        <v>749.87306919933</v>
+        <v>3039.25791166093</v>
       </c>
       <c r="D106" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B107" s="1" t="n">
-        <v>45817</v>
+        <v>45880</v>
       </c>
       <c r="C107" t="n">
-        <v>4412.64180269369</v>
+        <v>4775.20972744648</v>
       </c>
       <c r="D107" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B108" s="1" t="n">
-        <v>45826</v>
+        <v>45887</v>
       </c>
       <c r="C108" t="n">
-        <v>6968.33616394737</v>
+        <v>2089.81926332235</v>
       </c>
       <c r="D108" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B109" s="1" t="n">
-        <v>45835</v>
+        <v>45894</v>
       </c>
       <c r="C109" t="n">
-        <v>1687.73157419569</v>
+        <v>4752.47660961459</v>
       </c>
       <c r="D109" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B110" s="1" t="n">
-        <v>45842</v>
+        <v>45901</v>
       </c>
       <c r="C110" t="n">
-        <v>761.833024239517</v>
+        <v>1541.24223720587</v>
       </c>
       <c r="D110" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B111" s="1" t="n">
-        <v>45849</v>
+        <v>45908</v>
       </c>
       <c r="C111" t="n">
-        <v>2588.80886828618</v>
+        <v>1063.45963611384</v>
       </c>
       <c r="D111" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B112" s="1" t="n">
-        <v>45856</v>
+        <v>45912</v>
       </c>
       <c r="C112" t="n">
-        <v>3605.2695200209</v>
+        <v>940.00173894257</v>
       </c>
       <c r="D112" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B113" s="1" t="n">
-        <v>45863</v>
+        <v>45918</v>
       </c>
       <c r="C113" t="n">
-        <v>2464.37485564112</v>
+        <v>31.3335119250464</v>
       </c>
       <c r="D113" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B114" s="1" t="n">
-        <v>45873</v>
+        <v>45810</v>
       </c>
       <c r="C114" t="n">
-        <v>3566.94051479447</v>
+        <v>820.429289044661</v>
       </c>
       <c r="D114" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B115" s="1" t="n">
-        <v>45880</v>
+        <v>45817</v>
       </c>
       <c r="C115" t="n">
-        <v>5545.11780891709</v>
+        <v>4438.5887346754</v>
       </c>
       <c r="D115" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B116" s="1" t="n">
-        <v>45887</v>
+        <v>45826</v>
       </c>
       <c r="C116" t="n">
-        <v>2723.46038359217</v>
+        <v>3375.80821888685</v>
       </c>
       <c r="D116" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B117" s="1" t="n">
-        <v>45894</v>
+        <v>45835</v>
       </c>
       <c r="C117" t="n">
-        <v>3638.2311832252</v>
+        <v>783.186507035906</v>
       </c>
       <c r="D117" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B118" s="1" t="n">
-        <v>45901</v>
+        <v>45842</v>
       </c>
       <c r="C118" t="n">
-        <v>1849.60594842151</v>
+        <v>631.923814275014</v>
       </c>
       <c r="D118" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B119" s="1" t="n">
-        <v>45810</v>
+        <v>45849</v>
       </c>
       <c r="C119" t="n">
-        <v>654.622171815671</v>
+        <v>1315.52124698387</v>
       </c>
       <c r="D119" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B120" s="1" t="n">
-        <v>45817</v>
+        <v>45856</v>
       </c>
       <c r="C120" t="n">
-        <v>836.306701729539</v>
+        <v>2207.89437180403</v>
       </c>
       <c r="D120" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B121" s="1" t="n">
-        <v>45826</v>
+        <v>45863</v>
       </c>
       <c r="C121" t="n">
-        <v>752.809303565924</v>
+        <v>2258.29619366983</v>
       </c>
       <c r="D121" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B122" s="1" t="n">
-        <v>45835</v>
+        <v>45873</v>
       </c>
       <c r="C122" t="n">
-        <v>361.937925301449</v>
+        <v>3728.99958287456</v>
       </c>
       <c r="D122" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B123" s="1" t="n">
-        <v>45842</v>
+        <v>45880</v>
       </c>
       <c r="C123" t="n">
-        <v>274.147297459927</v>
+        <v>3912.32265691079</v>
       </c>
       <c r="D123" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B124" s="1" t="n">
-        <v>45849</v>
+        <v>45887</v>
       </c>
       <c r="C124" t="n">
-        <v>638.156969539091</v>
+        <v>3599.81922977165</v>
       </c>
       <c r="D124" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B125" s="1" t="n">
-        <v>45856</v>
+        <v>45894</v>
       </c>
       <c r="C125" t="n">
-        <v>671.100601945576</v>
+        <v>2913.7632567457</v>
       </c>
       <c r="D125" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B126" s="1" t="n">
-        <v>45863</v>
+        <v>45901</v>
       </c>
       <c r="C126" t="n">
-        <v>1126.92089194702</v>
+        <v>2488.12022404981</v>
       </c>
       <c r="D126" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B127" s="1" t="n">
-        <v>45873</v>
+        <v>45908</v>
       </c>
       <c r="C127" t="n">
-        <v>1904.69958425363</v>
+        <v>1047.56782225816</v>
       </c>
       <c r="D127" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B128" s="1" t="n">
-        <v>45880</v>
+        <v>45912</v>
       </c>
       <c r="C128" t="n">
-        <v>3800.93540490905</v>
+        <v>1336.84030216341</v>
       </c>
       <c r="D128" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B129" s="1" t="n">
-        <v>45887</v>
+        <v>45918</v>
       </c>
       <c r="C129" t="n">
-        <v>2170.9732688459</v>
+        <v>106.835647202663</v>
       </c>
       <c r="D129" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B130" s="1" t="n">
-        <v>45894</v>
+        <v>45810</v>
       </c>
       <c r="C130" t="n">
-        <v>3307.44136835169</v>
+        <v>749.87306919933</v>
       </c>
       <c r="D130" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B131" s="1" t="n">
-        <v>45901</v>
+        <v>45817</v>
       </c>
       <c r="C131" t="n">
-        <v>988.497215490608</v>
+        <v>4412.64180269369</v>
       </c>
       <c r="D131" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B132" s="1" t="n">
-        <v>45810</v>
+        <v>45826</v>
       </c>
       <c r="C132" t="n">
-        <v>714.089199892923</v>
+        <v>6968.33616394737</v>
       </c>
       <c r="D132" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B133" s="1" t="n">
-        <v>45817</v>
+        <v>45835</v>
       </c>
       <c r="C133" t="n">
-        <v>1332.31394460659</v>
+        <v>1687.73157419569</v>
       </c>
       <c r="D133" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B134" s="1" t="n">
-        <v>45826</v>
+        <v>45842</v>
       </c>
       <c r="C134" t="n">
-        <v>1403.48926864965</v>
+        <v>761.833024239517</v>
       </c>
       <c r="D134" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B135" s="1" t="n">
-        <v>45835</v>
+        <v>45849</v>
       </c>
       <c r="C135" t="n">
-        <v>423.584800449672</v>
+        <v>2588.80886828618</v>
       </c>
       <c r="D135" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B136" s="1" t="n">
-        <v>45842</v>
+        <v>45856</v>
       </c>
       <c r="C136" t="n">
-        <v>691.944631498715</v>
+        <v>3605.2695200209</v>
       </c>
       <c r="D136" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B137" s="1" t="n">
-        <v>45849</v>
+        <v>45863</v>
       </c>
       <c r="C137" t="n">
-        <v>1520.16740554049</v>
+        <v>2464.37485564112</v>
       </c>
       <c r="D137" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B138" s="1" t="n">
-        <v>45856</v>
+        <v>45873</v>
       </c>
       <c r="C138" t="n">
-        <v>1394.70386978331</v>
+        <v>3566.94051479447</v>
       </c>
       <c r="D138" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B139" s="1" t="n">
-        <v>45863</v>
+        <v>45880</v>
       </c>
       <c r="C139" t="n">
-        <v>1945.74582627245</v>
+        <v>5545.11780891709</v>
       </c>
       <c r="D139" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B140" s="1" t="n">
-        <v>45873</v>
+        <v>45887</v>
       </c>
       <c r="C140" t="n">
-        <v>2541.97761269932</v>
+        <v>2723.46038359217</v>
       </c>
       <c r="D140" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B141" s="1" t="n">
-        <v>45880</v>
+        <v>45894</v>
       </c>
       <c r="C141" t="n">
-        <v>3884.74955947511</v>
+        <v>3638.2311832252</v>
       </c>
       <c r="D141" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B142" s="1" t="n">
-        <v>45887</v>
+        <v>45901</v>
       </c>
       <c r="C142" t="n">
-        <v>1740.78269526192</v>
+        <v>1849.60594842151</v>
       </c>
       <c r="D142" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B143" s="1" t="n">
-        <v>45894</v>
+        <v>45908</v>
       </c>
       <c r="C143" t="n">
-        <v>2505.19645489012</v>
+        <v>2404.95349211011</v>
       </c>
       <c r="D143" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B144" s="1" t="n">
-        <v>45901</v>
+        <v>45912</v>
       </c>
       <c r="C144" t="n">
-        <v>973.643220252498</v>
+        <v>2923.99496976121</v>
       </c>
       <c r="D144" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B145" s="1" t="n">
-        <v>45810</v>
+        <v>45918</v>
       </c>
       <c r="C145" t="n">
-        <v>397.290437761417</v>
+        <v>30.5264686545068</v>
       </c>
       <c r="D145" t="s">
         <v>9</v>
@@ -2446,181 +2446,181 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B146" s="1" t="n">
-        <v>45817</v>
+        <v>45810</v>
       </c>
       <c r="C146" t="n">
-        <v>1926.90668700788</v>
+        <v>654.622171815671</v>
       </c>
       <c r="D146" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B147" s="1" t="n">
-        <v>45826</v>
+        <v>45817</v>
       </c>
       <c r="C147" t="n">
-        <v>3021.29841712424</v>
+        <v>836.306701729539</v>
       </c>
       <c r="D147" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B148" s="1" t="n">
-        <v>45835</v>
+        <v>45826</v>
       </c>
       <c r="C148" t="n">
-        <v>957.104912247124</v>
+        <v>752.809303565924</v>
       </c>
       <c r="D148" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B149" s="1" t="n">
-        <v>45842</v>
+        <v>45835</v>
       </c>
       <c r="C149" t="n">
-        <v>1649.6084629323</v>
+        <v>361.937925301449</v>
       </c>
       <c r="D149" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B150" s="1" t="n">
-        <v>45849</v>
+        <v>45842</v>
       </c>
       <c r="C150" t="n">
-        <v>1539.67899281552</v>
+        <v>274.147297459927</v>
       </c>
       <c r="D150" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B151" s="1" t="n">
-        <v>45856</v>
+        <v>45849</v>
       </c>
       <c r="C151" t="n">
-        <v>2459.63795093809</v>
+        <v>638.156969539091</v>
       </c>
       <c r="D151" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B152" s="1" t="n">
-        <v>45863</v>
+        <v>45856</v>
       </c>
       <c r="C152" t="n">
-        <v>1996.741477782</v>
+        <v>671.100601945576</v>
       </c>
       <c r="D152" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B153" s="1" t="n">
-        <v>45873</v>
+        <v>45863</v>
       </c>
       <c r="C153" t="n">
-        <v>3847.37405848995</v>
+        <v>1126.92089194702</v>
       </c>
       <c r="D153" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B154" s="1" t="n">
-        <v>45880</v>
+        <v>45873</v>
       </c>
       <c r="C154" t="n">
-        <v>2828.98818979552</v>
+        <v>1904.69958425363</v>
       </c>
       <c r="D154" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B155" s="1" t="n">
-        <v>45887</v>
+        <v>45880</v>
       </c>
       <c r="C155" t="n">
-        <v>2591.30540522796</v>
+        <v>3800.93540490905</v>
       </c>
       <c r="D155" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B156" s="1" t="n">
-        <v>45894</v>
+        <v>45887</v>
       </c>
       <c r="C156" t="n">
-        <v>1495.1664275966</v>
+        <v>2170.9732688459</v>
       </c>
       <c r="D156" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B157" s="1" t="n">
-        <v>45901</v>
+        <v>45894</v>
       </c>
       <c r="C157" t="n">
-        <v>1208.07345867435</v>
+        <v>3307.44136835169</v>
       </c>
       <c r="D157" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B158" s="1" t="n">
-        <v>45810</v>
+        <v>45901</v>
       </c>
       <c r="C158" t="n">
-        <v>564.435194569703</v>
+        <v>988.497215490608</v>
       </c>
       <c r="D158" t="s">
         <v>5</v>
@@ -2628,13 +2628,13 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B159" s="1" t="n">
-        <v>45817</v>
+        <v>45908</v>
       </c>
       <c r="C159" t="n">
-        <v>1545.70814869222</v>
+        <v>1157.73106587574</v>
       </c>
       <c r="D159" t="s">
         <v>5</v>
@@ -2642,13 +2642,13 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B160" s="1" t="n">
-        <v>45826</v>
+        <v>45912</v>
       </c>
       <c r="C160" t="n">
-        <v>3858.60188057439</v>
+        <v>898.830115935534</v>
       </c>
       <c r="D160" t="s">
         <v>5</v>
@@ -2656,13 +2656,13 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B161" s="1" t="n">
-        <v>45835</v>
+        <v>45918</v>
       </c>
       <c r="C161" t="n">
-        <v>75.8890033270052</v>
+        <v>10.4976730559286</v>
       </c>
       <c r="D161" t="s">
         <v>5</v>
@@ -2670,139 +2670,139 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B162" s="1" t="n">
-        <v>45842</v>
+        <v>45810</v>
       </c>
       <c r="C162" t="n">
-        <v>1607.81816898261</v>
+        <v>714.089199892923</v>
       </c>
       <c r="D162" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B163" s="1" t="n">
-        <v>45849</v>
+        <v>45817</v>
       </c>
       <c r="C163" t="n">
-        <v>651.305214716471</v>
+        <v>1332.31394460659</v>
       </c>
       <c r="D163" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B164" s="1" t="n">
-        <v>45856</v>
+        <v>45826</v>
       </c>
       <c r="C164" t="n">
-        <v>3182.90047392644</v>
+        <v>1403.48926864965</v>
       </c>
       <c r="D164" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B165" s="1" t="n">
-        <v>45863</v>
+        <v>45835</v>
       </c>
       <c r="C165" t="n">
-        <v>1054.40680471126</v>
+        <v>423.584800449672</v>
       </c>
       <c r="D165" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B166" s="1" t="n">
-        <v>45873</v>
+        <v>45842</v>
       </c>
       <c r="C166" t="n">
-        <v>3589.214407389</v>
+        <v>691.944631498715</v>
       </c>
       <c r="D166" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B167" s="1" t="n">
-        <v>45880</v>
+        <v>45849</v>
       </c>
       <c r="C167" t="n">
-        <v>2375.18299388371</v>
+        <v>1520.16740554049</v>
       </c>
       <c r="D167" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B168" s="1" t="n">
-        <v>45887</v>
+        <v>45856</v>
       </c>
       <c r="C168" t="n">
-        <v>2768.14096770644</v>
+        <v>1394.70386978331</v>
       </c>
       <c r="D168" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B169" s="1" t="n">
-        <v>45894</v>
+        <v>45863</v>
       </c>
       <c r="C169" t="n">
-        <v>1810.23398806605</v>
+        <v>1945.74582627245</v>
       </c>
       <c r="D169" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B170" s="1" t="n">
-        <v>45901</v>
+        <v>45873</v>
       </c>
       <c r="C170" t="n">
-        <v>2132.26773713034</v>
+        <v>2541.97761269932</v>
       </c>
       <c r="D170" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B171" s="1" t="n">
-        <v>45810</v>
+        <v>45880</v>
       </c>
       <c r="C171" t="n">
-        <v>447.392417911663</v>
+        <v>3884.74955947511</v>
       </c>
       <c r="D171" t="s">
         <v>7</v>
@@ -2810,13 +2810,13 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B172" s="1" t="n">
-        <v>45817</v>
+        <v>45887</v>
       </c>
       <c r="C172" t="n">
-        <v>2644.87800920049</v>
+        <v>1740.78269526192</v>
       </c>
       <c r="D172" t="s">
         <v>7</v>
@@ -2824,13 +2824,13 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B173" s="1" t="n">
-        <v>45826</v>
+        <v>45894</v>
       </c>
       <c r="C173" t="n">
-        <v>2858.8009710539</v>
+        <v>2505.19645489012</v>
       </c>
       <c r="D173" t="s">
         <v>7</v>
@@ -2838,13 +2838,13 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B174" s="1" t="n">
-        <v>45835</v>
+        <v>45901</v>
       </c>
       <c r="C174" t="n">
-        <v>763.112592784348</v>
+        <v>973.643220252498</v>
       </c>
       <c r="D174" t="s">
         <v>7</v>
@@ -2852,13 +2852,13 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B175" s="1" t="n">
-        <v>45842</v>
+        <v>45908</v>
       </c>
       <c r="C175" t="n">
-        <v>674.542028148127</v>
+        <v>929.750735529288</v>
       </c>
       <c r="D175" t="s">
         <v>7</v>
@@ -2866,13 +2866,13 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B176" s="1" t="n">
-        <v>45849</v>
+        <v>45912</v>
       </c>
       <c r="C176" t="n">
-        <v>1744.34596755931</v>
+        <v>863.428526988611</v>
       </c>
       <c r="D176" t="s">
         <v>7</v>
@@ -2880,13 +2880,13 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B177" s="1" t="n">
-        <v>45856</v>
+        <v>45918</v>
       </c>
       <c r="C177" t="n">
-        <v>1143.7372540643</v>
+        <v>31.4349107910936</v>
       </c>
       <c r="D177" t="s">
         <v>7</v>
@@ -2894,97 +2894,97 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B178" s="1" t="n">
-        <v>45863</v>
+        <v>45810</v>
       </c>
       <c r="C178" t="n">
-        <v>2601.30753317707</v>
+        <v>397.290437761417</v>
       </c>
       <c r="D178" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B179" s="1" t="n">
-        <v>45873</v>
+        <v>45817</v>
       </c>
       <c r="C179" t="n">
-        <v>2436.60825019887</v>
+        <v>1926.90668700788</v>
       </c>
       <c r="D179" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B180" s="1" t="n">
-        <v>45880</v>
+        <v>45826</v>
       </c>
       <c r="C180" t="n">
-        <v>3629.61304883485</v>
+        <v>3021.29841712424</v>
       </c>
       <c r="D180" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B181" s="1" t="n">
-        <v>45887</v>
+        <v>45835</v>
       </c>
       <c r="C181" t="n">
-        <v>2475.83592992463</v>
+        <v>957.104912247124</v>
       </c>
       <c r="D181" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B182" s="1" t="n">
-        <v>45894</v>
+        <v>45842</v>
       </c>
       <c r="C182" t="n">
-        <v>2279.65892583665</v>
+        <v>1649.6084629323</v>
       </c>
       <c r="D182" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B183" s="1" t="n">
-        <v>45901</v>
+        <v>45849</v>
       </c>
       <c r="C183" t="n">
-        <v>998.259977017587</v>
+        <v>1539.67899281552</v>
       </c>
       <c r="D183" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B184" s="1" t="n">
-        <v>45810</v>
+        <v>45856</v>
       </c>
       <c r="C184" t="n">
-        <v>844.462537825576</v>
+        <v>2459.63795093809</v>
       </c>
       <c r="D184" t="s">
         <v>9</v>
@@ -2992,13 +2992,13 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B185" s="1" t="n">
-        <v>45817</v>
+        <v>45863</v>
       </c>
       <c r="C185" t="n">
-        <v>2607.51843632838</v>
+        <v>1996.741477782</v>
       </c>
       <c r="D185" t="s">
         <v>9</v>
@@ -3006,13 +3006,13 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B186" s="1" t="n">
-        <v>45826</v>
+        <v>45873</v>
       </c>
       <c r="C186" t="n">
-        <v>1205.84904980573</v>
+        <v>3847.37405848995</v>
       </c>
       <c r="D186" t="s">
         <v>9</v>
@@ -3020,13 +3020,13 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B187" s="1" t="n">
-        <v>45835</v>
+        <v>45880</v>
       </c>
       <c r="C187" t="n">
-        <v>394.51261524864</v>
+        <v>2828.98818979552</v>
       </c>
       <c r="D187" t="s">
         <v>9</v>
@@ -3034,13 +3034,13 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B188" s="1" t="n">
-        <v>45842</v>
+        <v>45887</v>
       </c>
       <c r="C188" t="n">
-        <v>296.790183728622</v>
+        <v>2591.30540522796</v>
       </c>
       <c r="D188" t="s">
         <v>9</v>
@@ -3048,13 +3048,13 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B189" s="1" t="n">
-        <v>45849</v>
+        <v>45894</v>
       </c>
       <c r="C189" t="n">
-        <v>1029.40856752812</v>
+        <v>1495.1664275966</v>
       </c>
       <c r="D189" t="s">
         <v>9</v>
@@ -3062,13 +3062,13 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B190" s="1" t="n">
-        <v>45856</v>
+        <v>45901</v>
       </c>
       <c r="C190" t="n">
-        <v>822.899413189293</v>
+        <v>1208.07345867435</v>
       </c>
       <c r="D190" t="s">
         <v>9</v>
@@ -3076,13 +3076,13 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B191" s="1" t="n">
-        <v>45863</v>
+        <v>45908</v>
       </c>
       <c r="C191" t="n">
-        <v>1093.38451398619</v>
+        <v>1178.95542275766</v>
       </c>
       <c r="D191" t="s">
         <v>9</v>
@@ -3090,13 +3090,13 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B192" s="1" t="n">
-        <v>45873</v>
+        <v>45912</v>
       </c>
       <c r="C192" t="n">
-        <v>2628.07482556948</v>
+        <v>673.255967264892</v>
       </c>
       <c r="D192" t="s">
         <v>9</v>
@@ -3104,13 +3104,13 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B193" s="1" t="n">
-        <v>45880</v>
+        <v>45918</v>
       </c>
       <c r="C193" t="n">
-        <v>2995.86132481368</v>
+        <v>39.4795373586977</v>
       </c>
       <c r="D193" t="s">
         <v>9</v>
@@ -3118,43 +3118,673 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B194" s="1" t="n">
-        <v>45887</v>
+        <v>45810</v>
       </c>
       <c r="C194" t="n">
-        <v>2000.21497594218</v>
+        <v>564.435194569703</v>
       </c>
       <c r="D194" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B195" s="1" t="n">
-        <v>45894</v>
+        <v>45817</v>
       </c>
       <c r="C195" t="n">
-        <v>1879.36457990422</v>
+        <v>1545.70814869222</v>
       </c>
       <c r="D195" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="s">
+        <v>19</v>
+      </c>
+      <c r="B196" s="1" t="n">
+        <v>45826</v>
+      </c>
+      <c r="C196" t="n">
+        <v>3858.60188057439</v>
+      </c>
+      <c r="D196" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="s">
+        <v>19</v>
+      </c>
+      <c r="B197" s="1" t="n">
+        <v>45835</v>
+      </c>
+      <c r="C197" t="n">
+        <v>75.8890033270052</v>
+      </c>
+      <c r="D197" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="s">
+        <v>19</v>
+      </c>
+      <c r="B198" s="1" t="n">
+        <v>45842</v>
+      </c>
+      <c r="C198" t="n">
+        <v>1607.81816898261</v>
+      </c>
+      <c r="D198" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="s">
+        <v>19</v>
+      </c>
+      <c r="B199" s="1" t="n">
+        <v>45849</v>
+      </c>
+      <c r="C199" t="n">
+        <v>651.305214716471</v>
+      </c>
+      <c r="D199" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="s">
+        <v>19</v>
+      </c>
+      <c r="B200" s="1" t="n">
+        <v>45856</v>
+      </c>
+      <c r="C200" t="n">
+        <v>3182.90047392644</v>
+      </c>
+      <c r="D200" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="s">
+        <v>19</v>
+      </c>
+      <c r="B201" s="1" t="n">
+        <v>45863</v>
+      </c>
+      <c r="C201" t="n">
+        <v>1054.40680471126</v>
+      </c>
+      <c r="D201" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="s">
+        <v>19</v>
+      </c>
+      <c r="B202" s="1" t="n">
+        <v>45873</v>
+      </c>
+      <c r="C202" t="n">
+        <v>3589.214407389</v>
+      </c>
+      <c r="D202" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="s">
+        <v>19</v>
+      </c>
+      <c r="B203" s="1" t="n">
+        <v>45880</v>
+      </c>
+      <c r="C203" t="n">
+        <v>2375.18299388371</v>
+      </c>
+      <c r="D203" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="s">
+        <v>19</v>
+      </c>
+      <c r="B204" s="1" t="n">
+        <v>45887</v>
+      </c>
+      <c r="C204" t="n">
+        <v>2768.14096770644</v>
+      </c>
+      <c r="D204" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="s">
+        <v>19</v>
+      </c>
+      <c r="B205" s="1" t="n">
+        <v>45894</v>
+      </c>
+      <c r="C205" t="n">
+        <v>1810.23398806605</v>
+      </c>
+      <c r="D205" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="s">
+        <v>19</v>
+      </c>
+      <c r="B206" s="1" t="n">
+        <v>45901</v>
+      </c>
+      <c r="C206" t="n">
+        <v>2132.26773713034</v>
+      </c>
+      <c r="D206" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="s">
+        <v>19</v>
+      </c>
+      <c r="B207" s="1" t="n">
+        <v>45908</v>
+      </c>
+      <c r="C207" t="n">
+        <v>604.718699330132</v>
+      </c>
+      <c r="D207" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="s">
+        <v>19</v>
+      </c>
+      <c r="B208" s="1" t="n">
+        <v>45912</v>
+      </c>
+      <c r="C208" t="n">
+        <v>435.877350957814</v>
+      </c>
+      <c r="D208" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="s">
+        <v>19</v>
+      </c>
+      <c r="B209" s="1" t="n">
+        <v>45918</v>
+      </c>
+      <c r="C209" t="n">
+        <v>55.6387261658514</v>
+      </c>
+      <c r="D209" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="s">
+        <v>20</v>
+      </c>
+      <c r="B210" s="1" t="n">
+        <v>45810</v>
+      </c>
+      <c r="C210" t="n">
+        <v>447.392417911663</v>
+      </c>
+      <c r="D210" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="s">
+        <v>20</v>
+      </c>
+      <c r="B211" s="1" t="n">
+        <v>45817</v>
+      </c>
+      <c r="C211" t="n">
+        <v>2644.87800920049</v>
+      </c>
+      <c r="D211" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="s">
+        <v>20</v>
+      </c>
+      <c r="B212" s="1" t="n">
+        <v>45826</v>
+      </c>
+      <c r="C212" t="n">
+        <v>2858.8009710539</v>
+      </c>
+      <c r="D212" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="s">
+        <v>20</v>
+      </c>
+      <c r="B213" s="1" t="n">
+        <v>45835</v>
+      </c>
+      <c r="C213" t="n">
+        <v>763.112592784348</v>
+      </c>
+      <c r="D213" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="s">
+        <v>20</v>
+      </c>
+      <c r="B214" s="1" t="n">
+        <v>45842</v>
+      </c>
+      <c r="C214" t="n">
+        <v>674.542028148127</v>
+      </c>
+      <c r="D214" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="s">
+        <v>20</v>
+      </c>
+      <c r="B215" s="1" t="n">
+        <v>45849</v>
+      </c>
+      <c r="C215" t="n">
+        <v>1744.34596755931</v>
+      </c>
+      <c r="D215" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="s">
+        <v>20</v>
+      </c>
+      <c r="B216" s="1" t="n">
+        <v>45856</v>
+      </c>
+      <c r="C216" t="n">
+        <v>1143.7372540643</v>
+      </c>
+      <c r="D216" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="s">
+        <v>20</v>
+      </c>
+      <c r="B217" s="1" t="n">
+        <v>45863</v>
+      </c>
+      <c r="C217" t="n">
+        <v>2601.30753317707</v>
+      </c>
+      <c r="D217" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="s">
+        <v>20</v>
+      </c>
+      <c r="B218" s="1" t="n">
+        <v>45873</v>
+      </c>
+      <c r="C218" t="n">
+        <v>2436.60825019887</v>
+      </c>
+      <c r="D218" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="s">
+        <v>20</v>
+      </c>
+      <c r="B219" s="1" t="n">
+        <v>45880</v>
+      </c>
+      <c r="C219" t="n">
+        <v>3629.61304883485</v>
+      </c>
+      <c r="D219" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="s">
+        <v>20</v>
+      </c>
+      <c r="B220" s="1" t="n">
+        <v>45887</v>
+      </c>
+      <c r="C220" t="n">
+        <v>2475.83592992463</v>
+      </c>
+      <c r="D220" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="s">
+        <v>20</v>
+      </c>
+      <c r="B221" s="1" t="n">
+        <v>45894</v>
+      </c>
+      <c r="C221" t="n">
+        <v>2279.65892583665</v>
+      </c>
+      <c r="D221" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="s">
+        <v>20</v>
+      </c>
+      <c r="B222" s="1" t="n">
+        <v>45901</v>
+      </c>
+      <c r="C222" t="n">
+        <v>998.259977017587</v>
+      </c>
+      <c r="D222" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="s">
+        <v>20</v>
+      </c>
+      <c r="B223" s="1" t="n">
+        <v>45908</v>
+      </c>
+      <c r="C223" t="n">
+        <v>867.84005325841</v>
+      </c>
+      <c r="D223" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="s">
+        <v>20</v>
+      </c>
+      <c r="B224" s="1" t="n">
+        <v>45912</v>
+      </c>
+      <c r="C224" t="n">
+        <v>1313.90964847212</v>
+      </c>
+      <c r="D224" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="s">
+        <v>20</v>
+      </c>
+      <c r="B225" s="1" t="n">
+        <v>45918</v>
+      </c>
+      <c r="C225" t="n">
+        <v>30.7415294568651</v>
+      </c>
+      <c r="D225" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="s">
         <v>21</v>
       </c>
-      <c r="B196" s="1" t="n">
+      <c r="B226" s="1" t="n">
+        <v>45810</v>
+      </c>
+      <c r="C226" t="n">
+        <v>844.462537825576</v>
+      </c>
+      <c r="D226" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="s">
+        <v>21</v>
+      </c>
+      <c r="B227" s="1" t="n">
+        <v>45817</v>
+      </c>
+      <c r="C227" t="n">
+        <v>2607.51843632838</v>
+      </c>
+      <c r="D227" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="s">
+        <v>21</v>
+      </c>
+      <c r="B228" s="1" t="n">
+        <v>45826</v>
+      </c>
+      <c r="C228" t="n">
+        <v>1205.84904980573</v>
+      </c>
+      <c r="D228" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="s">
+        <v>21</v>
+      </c>
+      <c r="B229" s="1" t="n">
+        <v>45835</v>
+      </c>
+      <c r="C229" t="n">
+        <v>394.51261524864</v>
+      </c>
+      <c r="D229" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="s">
+        <v>21</v>
+      </c>
+      <c r="B230" s="1" t="n">
+        <v>45842</v>
+      </c>
+      <c r="C230" t="n">
+        <v>296.790183728622</v>
+      </c>
+      <c r="D230" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="s">
+        <v>21</v>
+      </c>
+      <c r="B231" s="1" t="n">
+        <v>45849</v>
+      </c>
+      <c r="C231" t="n">
+        <v>1029.40856752812</v>
+      </c>
+      <c r="D231" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="s">
+        <v>21</v>
+      </c>
+      <c r="B232" s="1" t="n">
+        <v>45856</v>
+      </c>
+      <c r="C232" t="n">
+        <v>822.899413189293</v>
+      </c>
+      <c r="D232" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="s">
+        <v>21</v>
+      </c>
+      <c r="B233" s="1" t="n">
+        <v>45863</v>
+      </c>
+      <c r="C233" t="n">
+        <v>1093.38451398619</v>
+      </c>
+      <c r="D233" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="s">
+        <v>21</v>
+      </c>
+      <c r="B234" s="1" t="n">
+        <v>45873</v>
+      </c>
+      <c r="C234" t="n">
+        <v>2628.07482556948</v>
+      </c>
+      <c r="D234" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="s">
+        <v>21</v>
+      </c>
+      <c r="B235" s="1" t="n">
+        <v>45880</v>
+      </c>
+      <c r="C235" t="n">
+        <v>2995.86132481368</v>
+      </c>
+      <c r="D235" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="s">
+        <v>21</v>
+      </c>
+      <c r="B236" s="1" t="n">
+        <v>45887</v>
+      </c>
+      <c r="C236" t="n">
+        <v>2000.21497594218</v>
+      </c>
+      <c r="D236" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="s">
+        <v>21</v>
+      </c>
+      <c r="B237" s="1" t="n">
+        <v>45894</v>
+      </c>
+      <c r="C237" t="n">
+        <v>1879.36457990422</v>
+      </c>
+      <c r="D237" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="s">
+        <v>21</v>
+      </c>
+      <c r="B238" s="1" t="n">
         <v>45901</v>
       </c>
-      <c r="C196" t="n">
+      <c r="C238" t="n">
         <v>967.384492520583</v>
       </c>
-      <c r="D196" t="s">
+      <c r="D238" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="s">
+        <v>21</v>
+      </c>
+      <c r="B239" s="1" t="n">
+        <v>45908</v>
+      </c>
+      <c r="C239" t="n">
+        <v>497.796936645038</v>
+      </c>
+      <c r="D239" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="s">
+        <v>21</v>
+      </c>
+      <c r="B240" s="1" t="n">
+        <v>45912</v>
+      </c>
+      <c r="C240" t="n">
+        <v>542.217662983649</v>
+      </c>
+      <c r="D240" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="s">
+        <v>21</v>
+      </c>
+      <c r="B241" s="1" t="n">
+        <v>45918</v>
+      </c>
+      <c r="C241" t="n">
+        <v>39.5592660515528</v>
+      </c>
+      <c r="D241" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>